<commit_message>
extração de dados do excel, modificação nas document_page, acréscimo do formato azimute/distância
</commit_message>
<xml_diff>
--- a/models/LAUDO DE AVALIAÇÃO N° 12941255 - MAURICIO MIYASAKI.xlsx
+++ b/models/LAUDO DE AVALIAÇÃO N° 12941255 - MAURICIO MIYASAKI.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="874" activeTab="3"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" tabRatio="874" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="CAPA DO LAUDO" sheetId="1" r:id="rId1"/>
@@ -2179,7 +2179,7 @@
     <xf numFmtId="9" fontId="39" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="462">
+  <cellXfs count="464">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="32" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2924,62 +2924,59 @@
     <xf numFmtId="0" fontId="55" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="10" fontId="63" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="63" fillId="0" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="54" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="54" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="54" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="55" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="55" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="55" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="63" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="63" fillId="0" borderId="14" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="54" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="52" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="54" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="54" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="54" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="55" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="169" fontId="46" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3093,20 +3090,20 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="170" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3126,13 +3123,13 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3218,6 +3215,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3247,9 +3247,6 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="9" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3409,6 +3406,11 @@
     <xf numFmtId="0" fontId="61" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="56" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hiperlink" xfId="4" builtinId="8"/>
@@ -4579,24 +4581,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="17.100000000000001" customHeight="1">
-      <c r="B1" s="437" t="s">
+      <c r="B1" s="436" t="s">
         <v>231</v>
       </c>
-      <c r="C1" s="438"/>
-      <c r="D1" s="438"/>
-      <c r="E1" s="438"/>
-      <c r="F1" s="438"/>
-      <c r="G1" s="438"/>
-      <c r="H1" s="439"/>
+      <c r="C1" s="437"/>
+      <c r="D1" s="437"/>
+      <c r="E1" s="437"/>
+      <c r="F1" s="437"/>
+      <c r="G1" s="437"/>
+      <c r="H1" s="438"/>
     </row>
     <row r="2" spans="2:12" ht="17.100000000000001" customHeight="1">
-      <c r="B2" s="433"/>
-      <c r="C2" s="434"/>
-      <c r="D2" s="434"/>
-      <c r="E2" s="434"/>
-      <c r="F2" s="434"/>
-      <c r="G2" s="434"/>
-      <c r="H2" s="435"/>
+      <c r="B2" s="432"/>
+      <c r="C2" s="433"/>
+      <c r="D2" s="433"/>
+      <c r="E2" s="433"/>
+      <c r="F2" s="433"/>
+      <c r="G2" s="433"/>
+      <c r="H2" s="434"/>
       <c r="K2" s="7"/>
       <c r="L2" s="8"/>
     </row>
@@ -4631,30 +4633,30 @@
       <c r="H5" s="55"/>
     </row>
     <row r="6" spans="2:12" s="10" customFormat="1" ht="12.75" customHeight="1">
-      <c r="B6" s="442" t="s">
+      <c r="B6" s="441" t="s">
         <v>259</v>
       </c>
-      <c r="C6" s="444" t="s">
+      <c r="C6" s="443" t="s">
         <v>260</v>
       </c>
-      <c r="D6" s="446" t="s">
+      <c r="D6" s="445" t="s">
         <v>261</v>
       </c>
-      <c r="E6" s="447" t="s">
+      <c r="E6" s="446" t="s">
         <v>262</v>
       </c>
-      <c r="F6" s="447" t="s">
+      <c r="F6" s="446" t="s">
         <v>263</v>
       </c>
-      <c r="G6" s="440" t="s">
+      <c r="G6" s="439" t="s">
         <v>264</v>
       </c>
-      <c r="H6" s="441"/>
+      <c r="H6" s="440"/>
     </row>
     <row r="7" spans="2:12" s="10" customFormat="1" ht="22.5" customHeight="1">
-      <c r="B7" s="443"/>
-      <c r="C7" s="445"/>
-      <c r="D7" s="445"/>
+      <c r="B7" s="442"/>
+      <c r="C7" s="444"/>
+      <c r="D7" s="444"/>
       <c r="E7" s="254"/>
       <c r="F7" s="254"/>
       <c r="G7" s="47" t="s">
@@ -4677,7 +4679,7 @@
       </c>
     </row>
     <row r="9" spans="2:12">
-      <c r="B9" s="448" t="s">
+      <c r="B9" s="447" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="243"/>
@@ -4702,30 +4704,30 @@
       <c r="H10" s="61"/>
     </row>
     <row r="11" spans="2:12" ht="12.75" customHeight="1">
-      <c r="B11" s="442" t="s">
+      <c r="B11" s="441" t="s">
         <v>259</v>
       </c>
-      <c r="C11" s="444" t="s">
+      <c r="C11" s="443" t="s">
         <v>260</v>
       </c>
-      <c r="D11" s="446" t="s">
+      <c r="D11" s="445" t="s">
         <v>261</v>
       </c>
-      <c r="E11" s="436" t="s">
+      <c r="E11" s="435" t="s">
         <v>267</v>
       </c>
-      <c r="F11" s="436" t="s">
+      <c r="F11" s="435" t="s">
         <v>263</v>
       </c>
-      <c r="G11" s="440" t="s">
+      <c r="G11" s="439" t="s">
         <v>264</v>
       </c>
-      <c r="H11" s="441"/>
+      <c r="H11" s="440"/>
     </row>
     <row r="12" spans="2:12" ht="22.5" customHeight="1">
-      <c r="B12" s="443"/>
-      <c r="C12" s="445"/>
-      <c r="D12" s="445"/>
+      <c r="B12" s="442"/>
+      <c r="C12" s="444"/>
+      <c r="D12" s="444"/>
       <c r="E12" s="254"/>
       <c r="F12" s="254"/>
       <c r="G12" s="47" t="s">
@@ -4748,7 +4750,7 @@
       </c>
     </row>
     <row r="14" spans="2:12">
-      <c r="B14" s="448" t="s">
+      <c r="B14" s="447" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="243"/>
@@ -4773,30 +4775,30 @@
       <c r="H15" s="53"/>
     </row>
     <row r="16" spans="2:12" ht="12.75" customHeight="1">
-      <c r="B16" s="442" t="s">
+      <c r="B16" s="441" t="s">
         <v>259</v>
       </c>
-      <c r="C16" s="444" t="s">
+      <c r="C16" s="443" t="s">
         <v>269</v>
       </c>
-      <c r="D16" s="446" t="s">
+      <c r="D16" s="445" t="s">
         <v>261</v>
       </c>
-      <c r="E16" s="436" t="s">
+      <c r="E16" s="435" t="s">
         <v>267</v>
       </c>
-      <c r="F16" s="436" t="s">
+      <c r="F16" s="435" t="s">
         <v>263</v>
       </c>
-      <c r="G16" s="440" t="s">
+      <c r="G16" s="439" t="s">
         <v>264</v>
       </c>
-      <c r="H16" s="441"/>
+      <c r="H16" s="440"/>
     </row>
     <row r="17" spans="2:8" ht="21" customHeight="1">
-      <c r="B17" s="443"/>
-      <c r="C17" s="445"/>
-      <c r="D17" s="445"/>
+      <c r="B17" s="442"/>
+      <c r="C17" s="444"/>
+      <c r="D17" s="444"/>
       <c r="E17" s="254"/>
       <c r="F17" s="254"/>
       <c r="G17" s="22" t="s">
@@ -4821,7 +4823,7 @@
       </c>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="448" t="s">
+      <c r="B19" s="447" t="s">
         <v>20</v>
       </c>
       <c r="C19" s="243"/>
@@ -4846,30 +4848,30 @@
       <c r="H20" s="53"/>
     </row>
     <row r="21" spans="2:8" ht="12.75" customHeight="1">
-      <c r="B21" s="442" t="s">
+      <c r="B21" s="441" t="s">
         <v>259</v>
       </c>
-      <c r="C21" s="444" t="s">
+      <c r="C21" s="443" t="s">
         <v>260</v>
       </c>
-      <c r="D21" s="446" t="s">
+      <c r="D21" s="445" t="s">
         <v>261</v>
       </c>
-      <c r="E21" s="436" t="s">
+      <c r="E21" s="435" t="s">
         <v>267</v>
       </c>
-      <c r="F21" s="436" t="s">
+      <c r="F21" s="435" t="s">
         <v>263</v>
       </c>
-      <c r="G21" s="440" t="s">
+      <c r="G21" s="439" t="s">
         <v>264</v>
       </c>
-      <c r="H21" s="441"/>
+      <c r="H21" s="440"/>
     </row>
     <row r="22" spans="2:8" ht="21.75" customHeight="1">
-      <c r="B22" s="443"/>
-      <c r="C22" s="445"/>
-      <c r="D22" s="445"/>
+      <c r="B22" s="442"/>
+      <c r="C22" s="444"/>
+      <c r="D22" s="444"/>
       <c r="E22" s="254"/>
       <c r="F22" s="254"/>
       <c r="G22" s="47" t="s">
@@ -4892,14 +4894,14 @@
       </c>
     </row>
     <row r="24" spans="2:8" ht="13.5" customHeight="1" thickBot="1">
-      <c r="B24" s="431" t="s">
+      <c r="B24" s="430" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="432"/>
-      <c r="D24" s="432"/>
-      <c r="E24" s="432"/>
-      <c r="F24" s="432"/>
-      <c r="G24" s="381"/>
+      <c r="C24" s="431"/>
+      <c r="D24" s="431"/>
+      <c r="E24" s="431"/>
+      <c r="F24" s="431"/>
+      <c r="G24" s="380"/>
       <c r="H24" s="66"/>
     </row>
   </sheetData>
@@ -4959,14 +4961,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" s="1" customFormat="1" ht="17.100000000000001" customHeight="1">
-      <c r="B1" s="451" t="s">
+      <c r="B1" s="450" t="s">
         <v>231</v>
       </c>
-      <c r="C1" s="434"/>
-      <c r="D1" s="434"/>
-      <c r="E1" s="434"/>
-      <c r="F1" s="434"/>
-      <c r="G1" s="434"/>
+      <c r="C1" s="433"/>
+      <c r="D1" s="433"/>
+      <c r="E1" s="433"/>
+      <c r="F1" s="433"/>
+      <c r="G1" s="433"/>
       <c r="H1" s="41"/>
       <c r="I1" s="41"/>
     </row>
@@ -4990,7 +4992,7 @@
       <c r="I3" s="5"/>
     </row>
     <row r="4" spans="2:13" ht="13.5" customHeight="1">
-      <c r="B4" s="452" t="s">
+      <c r="B4" s="451" t="s">
         <v>272</v>
       </c>
       <c r="C4" s="243"/>
@@ -5001,19 +5003,19 @@
       <c r="H4" s="27"/>
     </row>
     <row r="5" spans="2:13">
-      <c r="B5" s="453" t="s">
+      <c r="B5" s="452" t="s">
         <v>273</v>
       </c>
-      <c r="C5" s="449" t="s">
+      <c r="C5" s="448" t="s">
         <v>274</v>
       </c>
-      <c r="D5" s="449" t="s">
+      <c r="D5" s="448" t="s">
         <v>275</v>
       </c>
-      <c r="E5" s="449" t="s">
+      <c r="E5" s="448" t="s">
         <v>276</v>
       </c>
-      <c r="F5" s="450" t="s">
+      <c r="F5" s="449" t="s">
         <v>277</v>
       </c>
       <c r="G5" s="243"/>
@@ -5021,9 +5023,9 @@
     </row>
     <row r="6" spans="2:13">
       <c r="B6" s="254"/>
-      <c r="C6" s="445"/>
-      <c r="D6" s="445"/>
-      <c r="E6" s="445"/>
+      <c r="C6" s="444"/>
+      <c r="D6" s="444"/>
+      <c r="E6" s="444"/>
       <c r="F6" s="30" t="s">
         <v>265</v>
       </c>
@@ -5075,7 +5077,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="15" customHeight="1">
-      <c r="A1" s="461" t="s">
+      <c r="A1" s="460" t="s">
         <v>7</v>
       </c>
       <c r="B1" s="248"/>
@@ -5091,18 +5093,18 @@
       <c r="L1" s="248"/>
       <c r="M1" s="248"/>
       <c r="N1" s="248"/>
-      <c r="O1" s="454"/>
+      <c r="O1" s="453"/>
       <c r="P1" s="248"/>
       <c r="Q1" s="248"/>
       <c r="R1" s="248"/>
       <c r="S1" s="248"/>
     </row>
     <row r="2" spans="1:19" ht="15" customHeight="1">
-      <c r="A2" s="459" t="s">
+      <c r="A2" s="458" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="248"/>
-      <c r="C2" s="459" t="s">
+      <c r="C2" s="458" t="s">
         <v>278</v>
       </c>
       <c r="D2" s="248"/>
@@ -5111,7 +5113,7 @@
       <c r="G2" s="248"/>
       <c r="H2" s="248"/>
       <c r="I2" s="248"/>
-      <c r="J2" s="460" t="s">
+      <c r="J2" s="459" t="s">
         <v>279</v>
       </c>
       <c r="K2" s="248"/>
@@ -5120,11 +5122,11 @@
       <c r="O2" s="239"/>
     </row>
     <row r="3" spans="1:19" ht="15" customHeight="1">
-      <c r="A3" s="456" t="s">
+      <c r="A3" s="455" t="s">
         <v>280</v>
       </c>
       <c r="B3" s="248"/>
-      <c r="C3" s="456" t="s">
+      <c r="C3" s="455" t="s">
         <v>278</v>
       </c>
       <c r="D3" s="248"/>
@@ -5133,7 +5135,7 @@
       <c r="G3" s="248"/>
       <c r="H3" s="248"/>
       <c r="I3" s="248"/>
-      <c r="J3" s="456" t="s">
+      <c r="J3" s="455" t="s">
         <v>281</v>
       </c>
       <c r="K3" s="248"/>
@@ -5142,11 +5144,11 @@
       <c r="N3" s="248"/>
     </row>
     <row r="4" spans="1:19" ht="15" customHeight="1">
-      <c r="A4" s="456" t="s">
+      <c r="A4" s="455" t="s">
         <v>282</v>
       </c>
       <c r="B4" s="248"/>
-      <c r="C4" s="456" t="s">
+      <c r="C4" s="455" t="s">
         <v>283</v>
       </c>
       <c r="D4" s="248"/>
@@ -5155,18 +5157,18 @@
       <c r="G4" s="248"/>
       <c r="H4" s="248"/>
       <c r="I4" s="248"/>
-      <c r="J4" s="458"/>
+      <c r="J4" s="457"/>
       <c r="K4" s="248"/>
       <c r="L4" s="248"/>
       <c r="M4" s="248"/>
       <c r="N4" s="248"/>
     </row>
     <row r="5" spans="1:19" ht="15" customHeight="1">
-      <c r="A5" s="456" t="s">
+      <c r="A5" s="455" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="248"/>
-      <c r="C5" s="456" t="s">
+      <c r="C5" s="455" t="s">
         <v>284</v>
       </c>
       <c r="D5" s="248"/>
@@ -5175,18 +5177,18 @@
       <c r="G5" s="248"/>
       <c r="H5" s="248"/>
       <c r="I5" s="248"/>
-      <c r="J5" s="458"/>
+      <c r="J5" s="457"/>
       <c r="K5" s="248"/>
       <c r="L5" s="248"/>
       <c r="M5" s="248"/>
       <c r="N5" s="248"/>
     </row>
     <row r="6" spans="1:19" ht="15" customHeight="1">
-      <c r="A6" s="456" t="s">
+      <c r="A6" s="455" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="248"/>
-      <c r="C6" s="456" t="s">
+      <c r="C6" s="455" t="s">
         <v>285</v>
       </c>
       <c r="D6" s="248"/>
@@ -5195,7 +5197,7 @@
       <c r="G6" s="248"/>
       <c r="H6" s="248"/>
       <c r="I6" s="248"/>
-      <c r="J6" s="456" t="s">
+      <c r="J6" s="455" t="s">
         <v>286</v>
       </c>
       <c r="K6" s="248"/>
@@ -5204,7 +5206,7 @@
       <c r="N6" s="248"/>
     </row>
     <row r="7" spans="1:19" ht="15" customHeight="1">
-      <c r="A7" s="455" t="s">
+      <c r="A7" s="454" t="s">
         <v>287</v>
       </c>
       <c r="B7" s="248"/>
@@ -5245,7 +5247,7 @@
     <row r="29" spans="1:14" ht="15" customHeight="1"/>
     <row r="30" spans="1:14" ht="15" customHeight="1"/>
     <row r="31" spans="1:14" ht="15" customHeight="1">
-      <c r="A31" s="455" t="s">
+      <c r="A31" s="454" t="s">
         <v>288</v>
       </c>
       <c r="B31" s="248"/>
@@ -5263,22 +5265,22 @@
       <c r="N31" s="248"/>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1">
-      <c r="A32" s="457" t="s">
+      <c r="A32" s="456" t="s">
         <v>11</v>
       </c>
       <c r="B32" s="248"/>
       <c r="C32" s="248"/>
-      <c r="D32" s="457" t="s">
+      <c r="D32" s="456" t="s">
         <v>12</v>
       </c>
       <c r="E32" s="248"/>
       <c r="F32" s="248"/>
-      <c r="G32" s="457" t="s">
+      <c r="G32" s="456" t="s">
         <v>289</v>
       </c>
       <c r="H32" s="248"/>
       <c r="I32" s="248"/>
-      <c r="J32" s="457" t="s">
+      <c r="J32" s="456" t="s">
         <v>14</v>
       </c>
       <c r="K32" s="248"/>
@@ -5286,22 +5288,22 @@
       <c r="M32" s="248"/>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1">
-      <c r="A33" s="457" t="s">
+      <c r="A33" s="456" t="s">
         <v>290</v>
       </c>
       <c r="B33" s="248"/>
       <c r="C33" s="248"/>
-      <c r="D33" s="457" t="s">
+      <c r="D33" s="456" t="s">
         <v>291</v>
       </c>
       <c r="E33" s="248"/>
       <c r="F33" s="248"/>
-      <c r="G33" s="457" t="s">
+      <c r="G33" s="456" t="s">
         <v>292</v>
       </c>
       <c r="H33" s="248"/>
       <c r="I33" s="248"/>
-      <c r="J33" s="457" t="s">
+      <c r="J33" s="456" t="s">
         <v>293</v>
       </c>
       <c r="K33" s="248"/>
@@ -5309,7 +5311,7 @@
       <c r="M33" s="248"/>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1">
-      <c r="A34" s="455" t="s">
+      <c r="A34" s="454" t="s">
         <v>16</v>
       </c>
       <c r="B34" s="248"/>
@@ -5327,34 +5329,34 @@
       <c r="N34" s="248"/>
     </row>
     <row r="35" spans="1:14" ht="15" customHeight="1">
-      <c r="A35" s="457" t="s">
+      <c r="A35" s="456" t="s">
         <v>11</v>
       </c>
       <c r="B35" s="248"/>
       <c r="C35" s="248"/>
-      <c r="F35" s="457" t="s">
+      <c r="F35" s="456" t="s">
         <v>294</v>
       </c>
       <c r="G35" s="248"/>
       <c r="H35" s="248"/>
-      <c r="K35" s="457" t="s">
+      <c r="K35" s="456" t="s">
         <v>295</v>
       </c>
       <c r="L35" s="248"/>
       <c r="M35" s="248"/>
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1">
-      <c r="A36" s="457" t="s">
+      <c r="A36" s="456" t="s">
         <v>290</v>
       </c>
       <c r="B36" s="248"/>
       <c r="C36" s="248"/>
-      <c r="F36" s="457" t="s">
+      <c r="F36" s="456" t="s">
         <v>296</v>
       </c>
       <c r="G36" s="248"/>
       <c r="H36" s="248"/>
-      <c r="K36" s="457" t="s">
+      <c r="K36" s="456" t="s">
         <v>297</v>
       </c>
       <c r="L36" s="248"/>
@@ -5728,19 +5730,19 @@
       <c r="T4" s="207"/>
     </row>
     <row r="5" spans="3:20">
-      <c r="C5" s="293" t="s">
+      <c r="C5" s="295" t="s">
         <v>61</v>
       </c>
       <c r="D5" s="254"/>
-      <c r="E5" s="293" t="s">
+      <c r="E5" s="295" t="s">
         <v>62</v>
       </c>
       <c r="F5" s="254"/>
-      <c r="G5" s="293" t="s">
+      <c r="G5" s="295" t="s">
         <v>63</v>
       </c>
       <c r="H5" s="254"/>
-      <c r="I5" s="297" t="s">
+      <c r="I5" s="293" t="s">
         <v>64</v>
       </c>
       <c r="J5" s="254"/>
@@ -5770,7 +5772,7 @@
         <v>67</v>
       </c>
       <c r="H6" s="244"/>
-      <c r="I6" s="300" t="s">
+      <c r="I6" s="297" t="s">
         <v>67</v>
       </c>
       <c r="J6" s="244"/>
@@ -5858,7 +5860,7 @@
         <v>80</v>
       </c>
       <c r="H9" s="244"/>
-      <c r="I9" s="300">
+      <c r="I9" s="297">
         <v>0.65039999999999998</v>
       </c>
       <c r="J9" s="244"/>
@@ -5942,21 +5944,21 @@
         <v>77</v>
       </c>
       <c r="H13" s="244"/>
-      <c r="I13" s="300" t="s">
+      <c r="I13" s="297" t="s">
         <v>78</v>
       </c>
       <c r="J13" s="244"/>
     </row>
     <row r="16" spans="3:20">
-      <c r="C16" s="298" t="s">
+      <c r="C16" s="461" t="s">
         <v>302</v>
       </c>
-      <c r="D16" s="243"/>
-      <c r="E16" s="243"/>
-      <c r="F16" s="243"/>
-      <c r="G16" s="243"/>
-      <c r="H16" s="243"/>
-      <c r="I16" s="244"/>
+      <c r="D16" s="462"/>
+      <c r="E16" s="462"/>
+      <c r="F16" s="462"/>
+      <c r="G16" s="462"/>
+      <c r="H16" s="462"/>
+      <c r="I16" s="463"/>
     </row>
     <row r="17" spans="3:10">
       <c r="C17" s="281" t="s">
@@ -5974,24 +5976,24 @@
       <c r="I17" s="244"/>
     </row>
     <row r="18" spans="3:10" ht="15">
-      <c r="C18" s="306" t="s">
+      <c r="C18" s="303" t="s">
         <v>304</v>
       </c>
-      <c r="D18" s="307"/>
-      <c r="E18" s="308"/>
-      <c r="F18" s="291">
+      <c r="D18" s="304"/>
+      <c r="E18" s="305"/>
+      <c r="F18" s="307">
         <f>AMOSTRAS!E11</f>
         <v>7.23</v>
       </c>
-      <c r="G18" s="292"/>
-      <c r="H18" s="295">
+      <c r="G18" s="308"/>
+      <c r="H18" s="291">
         <f>F18/C6</f>
         <v>0.13894681008488632</v>
       </c>
-      <c r="I18" s="296"/>
+      <c r="I18" s="292"/>
     </row>
     <row r="19" spans="3:10">
-      <c r="C19" s="309" t="s">
+      <c r="C19" s="306" t="s">
         <v>301</v>
       </c>
       <c r="D19" s="243"/>
@@ -6001,7 +6003,7 @@
         <v>24.851099999999999</v>
       </c>
       <c r="G19" s="244"/>
-      <c r="H19" s="299">
+      <c r="H19" s="296">
         <f>AMOSTRAS!F12</f>
         <v>0.4775907430291173</v>
       </c>
@@ -6013,19 +6015,19 @@
       </c>
       <c r="D20" s="289"/>
       <c r="E20" s="290"/>
-      <c r="F20" s="304">
+      <c r="F20" s="301">
         <f>AMOSTRAS!E13</f>
         <v>19.953199999999999</v>
       </c>
-      <c r="G20" s="305"/>
-      <c r="H20" s="302">
+      <c r="G20" s="302"/>
+      <c r="H20" s="299">
         <f>AMOSTRAS!F13</f>
         <v>0.38346244688599634</v>
       </c>
-      <c r="I20" s="303"/>
+      <c r="I20" s="300"/>
     </row>
     <row r="21" spans="3:10">
-      <c r="C21" s="301" t="s">
+      <c r="C21" s="298" t="s">
         <v>83</v>
       </c>
       <c r="D21" s="243"/>
@@ -6035,7 +6037,7 @@
         <v>52.034300000000002</v>
       </c>
       <c r="G21" s="244"/>
-      <c r="H21" s="299">
+      <c r="H21" s="296">
         <f>SUM(H18:I20)</f>
         <v>1</v>
       </c>
@@ -6044,7 +6046,6 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="G12:H12"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="I6:J6"/>
@@ -6060,6 +6061,13 @@
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="C16:I16"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="E12:F12"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="E5:F5"/>
@@ -6068,13 +6076,7 @@
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="E11:F11"/>
     <mergeCell ref="G5:H5"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="C16:I16"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
     <mergeCell ref="C4:J4"/>
     <mergeCell ref="C10:J10"/>
     <mergeCell ref="F21:G21"/>
@@ -6093,7 +6095,7 @@
     <mergeCell ref="C20:E20"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6118,7 +6120,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:14" ht="15" customHeight="1">
-      <c r="B3" s="328" t="s">
+      <c r="B3" s="327" t="s">
         <v>84</v>
       </c>
       <c r="C3" s="279"/>
@@ -6128,25 +6130,25 @@
       <c r="G3" s="279"/>
       <c r="H3" s="279"/>
       <c r="I3" s="279"/>
-      <c r="L3" s="371" t="s">
+      <c r="L3" s="370" t="s">
         <v>85</v>
       </c>
       <c r="M3" s="244"/>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1">
-      <c r="B4" s="320" t="s">
+      <c r="B4" s="319" t="s">
         <v>86</v>
       </c>
-      <c r="C4" s="321"/>
-      <c r="D4" s="321"/>
-      <c r="E4" s="373" t="s">
+      <c r="C4" s="320"/>
+      <c r="D4" s="320"/>
+      <c r="E4" s="372" t="s">
         <v>298</v>
       </c>
       <c r="F4" s="279"/>
       <c r="G4" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H4" s="341" t="s">
+      <c r="H4" s="340" t="s">
         <v>299</v>
       </c>
       <c r="I4" s="258"/>
@@ -6160,19 +6162,19 @@
       </c>
     </row>
     <row r="5" spans="2:14" ht="15" customHeight="1">
-      <c r="B5" s="318" t="s">
+      <c r="B5" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C5" s="279"/>
       <c r="D5" s="279"/>
-      <c r="E5" s="335" t="s">
+      <c r="E5" s="334" t="s">
         <v>90</v>
       </c>
       <c r="F5" s="279"/>
       <c r="G5" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H5" s="341" t="s">
+      <c r="H5" s="340" t="s">
         <v>49</v>
       </c>
       <c r="I5" s="258"/>
@@ -6185,56 +6187,56 @@
       </c>
     </row>
     <row r="6" spans="2:14" ht="15" customHeight="1">
-      <c r="B6" s="318" t="s">
+      <c r="B6" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C6" s="279"/>
       <c r="D6" s="279"/>
-      <c r="E6" s="351">
+      <c r="E6" s="359">
         <v>52.034300000000002</v>
       </c>
       <c r="F6" s="279"/>
       <c r="G6" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H6" s="346" t="s">
+      <c r="H6" s="345" t="s">
         <v>300</v>
       </c>
       <c r="I6" s="258"/>
     </row>
     <row r="7" spans="2:14" ht="15" customHeight="1">
       <c r="B7" s="165"/>
-      <c r="C7" s="334" t="s">
+      <c r="C7" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D7" s="279"/>
-      <c r="E7" s="353" t="s">
+      <c r="E7" s="352" t="s">
         <v>136</v>
       </c>
       <c r="F7" s="279"/>
       <c r="G7" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H7" s="317">
+      <c r="H7" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I7" s="258"/>
     </row>
     <row r="8" spans="2:14" ht="15" customHeight="1">
       <c r="B8" s="165"/>
-      <c r="C8" s="334" t="s">
+      <c r="C8" s="333" t="s">
         <v>99</v>
       </c>
       <c r="D8" s="279"/>
-      <c r="E8" s="360">
+      <c r="E8" s="358">
         <v>11173</v>
       </c>
       <c r="F8" s="279"/>
       <c r="G8" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H8" s="336"/>
+      <c r="H8" s="335"/>
       <c r="I8" s="258"/>
       <c r="J8" s="226"/>
       <c r="K8" s="226"/>
@@ -6243,7 +6245,7 @@
       <c r="N8" s="226"/>
     </row>
     <row r="9" spans="2:14" ht="15" customHeight="1">
-      <c r="B9" s="324" t="s">
+      <c r="B9" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C9" s="279"/>
@@ -6260,7 +6262,7 @@
       <c r="N9" s="226"/>
     </row>
     <row r="10" spans="2:14" ht="15" customHeight="1">
-      <c r="B10" s="333" t="s">
+      <c r="B10" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C10" s="279"/>
@@ -6271,7 +6273,7 @@
       <c r="F10" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G10" s="325" t="s">
+      <c r="G10" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H10" s="279"/>
@@ -6283,11 +6285,11 @@
       <c r="N10" s="226"/>
     </row>
     <row r="11" spans="2:14" ht="15" customHeight="1">
-      <c r="B11" s="368" t="s">
+      <c r="B11" s="367" t="s">
         <v>106</v>
       </c>
-      <c r="C11" s="369"/>
-      <c r="D11" s="369"/>
+      <c r="C11" s="368"/>
+      <c r="D11" s="368"/>
       <c r="E11" s="240">
         <v>7.23</v>
       </c>
@@ -6295,10 +6297,10 @@
         <f>E11/E6</f>
         <v>0.13894681008488632</v>
       </c>
-      <c r="G11" s="370">
+      <c r="G11" s="369">
         <v>1</v>
       </c>
-      <c r="H11" s="370"/>
+      <c r="H11" s="369"/>
       <c r="I11" s="167"/>
       <c r="J11" s="226"/>
       <c r="K11" s="226"/>
@@ -6307,7 +6309,7 @@
       <c r="N11" s="226"/>
     </row>
     <row r="12" spans="2:14" ht="15" customHeight="1">
-      <c r="B12" s="359" t="s">
+      <c r="B12" s="357" t="s">
         <v>117</v>
       </c>
       <c r="C12" s="279"/>
@@ -6320,7 +6322,7 @@
         <f>E12/E6</f>
         <v>0.4775907430291173</v>
       </c>
-      <c r="G12" s="314">
+      <c r="G12" s="313">
         <v>0.8</v>
       </c>
       <c r="H12" s="279"/>
@@ -6332,7 +6334,7 @@
       <c r="N12" s="226"/>
     </row>
     <row r="13" spans="2:14" ht="15" customHeight="1">
-      <c r="B13" s="354" t="s">
+      <c r="B13" s="353" t="s">
         <v>107</v>
       </c>
       <c r="C13" s="279"/>
@@ -6345,7 +6347,7 @@
         <f>E13/E6</f>
         <v>0.38346244688599634</v>
       </c>
-      <c r="G13" s="314">
+      <c r="G13" s="313">
         <v>0.6</v>
       </c>
       <c r="H13" s="279"/>
@@ -6361,7 +6363,7 @@
       <c r="N13" s="226"/>
     </row>
     <row r="14" spans="2:14" ht="15" customHeight="1">
-      <c r="B14" s="319" t="s">
+      <c r="B14" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C14" s="246"/>
@@ -6374,7 +6376,7 @@
         <f>SUM(F11:F13)</f>
         <v>1</v>
       </c>
-      <c r="G14" s="310">
+      <c r="G14" s="309">
         <f>(F12*G12)+(F13*G13)+F11*G11</f>
         <v>0.75109687263977798</v>
       </c>
@@ -6402,7 +6404,7 @@
       <c r="N15" s="226"/>
     </row>
     <row r="16" spans="2:14" ht="15" customHeight="1">
-      <c r="B16" s="328" t="s">
+      <c r="B16" s="327" t="s">
         <v>108</v>
       </c>
       <c r="C16" s="279"/>
@@ -6415,19 +6417,19 @@
       <c r="K16" s="203"/>
     </row>
     <row r="17" spans="2:11" ht="15" customHeight="1">
-      <c r="B17" s="320" t="s">
+      <c r="B17" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="321"/>
-      <c r="D17" s="321"/>
-      <c r="E17" s="312" t="s">
+      <c r="C17" s="320"/>
+      <c r="D17" s="320"/>
+      <c r="E17" s="311" t="s">
         <v>110</v>
       </c>
       <c r="F17" s="279"/>
       <c r="G17" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H17" s="342" t="s">
+      <c r="H17" s="341" t="s">
         <v>111</v>
       </c>
       <c r="I17" s="258"/>
@@ -6436,31 +6438,31 @@
       </c>
     </row>
     <row r="18" spans="2:11" ht="15" customHeight="1">
-      <c r="B18" s="318" t="s">
+      <c r="B18" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C18" s="279"/>
       <c r="D18" s="279"/>
-      <c r="E18" s="335" t="s">
+      <c r="E18" s="334" t="s">
         <v>90</v>
       </c>
       <c r="F18" s="279"/>
       <c r="G18" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H18" s="345" t="s">
+      <c r="H18" s="344" t="s">
         <v>49</v>
       </c>
       <c r="I18" s="258"/>
       <c r="K18" s="203"/>
     </row>
     <row r="19" spans="2:11" ht="15" customHeight="1">
-      <c r="B19" s="318" t="s">
+      <c r="B19" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C19" s="279"/>
       <c r="D19" s="279"/>
-      <c r="E19" s="352">
+      <c r="E19" s="351">
         <f>3500*4.84</f>
         <v>16940</v>
       </c>
@@ -6468,18 +6470,18 @@
       <c r="G19" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H19" s="315" t="s">
+      <c r="H19" s="314" t="s">
         <v>95</v>
       </c>
       <c r="I19" s="258"/>
     </row>
     <row r="20" spans="2:11" ht="15" customHeight="1">
       <c r="B20" s="211"/>
-      <c r="C20" s="334" t="s">
+      <c r="C20" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D20" s="279"/>
-      <c r="E20" s="340">
+      <c r="E20" s="339">
         <f>180000000</f>
         <v>180000000</v>
       </c>
@@ -6487,7 +6489,7 @@
       <c r="G20" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H20" s="316">
+      <c r="H20" s="315">
         <f>E20/E19</f>
         <v>10625.737898465171</v>
       </c>
@@ -6499,42 +6501,42 @@
     </row>
     <row r="21" spans="2:11" ht="15" customHeight="1">
       <c r="B21" s="212"/>
-      <c r="C21" s="334" t="s">
+      <c r="C21" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D21" s="279"/>
-      <c r="E21" s="356" t="s">
+      <c r="E21" s="355" t="s">
         <v>116</v>
       </c>
       <c r="F21" s="279"/>
       <c r="G21" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H21" s="317">
+      <c r="H21" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I21" s="258"/>
     </row>
     <row r="22" spans="2:11" ht="15" customHeight="1">
       <c r="B22" s="212"/>
-      <c r="C22" s="334" t="s">
+      <c r="C22" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D22" s="279"/>
-      <c r="E22" s="312" t="s">
+      <c r="E22" s="311" t="s">
         <v>97</v>
       </c>
       <c r="F22" s="279"/>
       <c r="G22" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H22" s="348"/>
+      <c r="H22" s="346"/>
       <c r="I22" s="258"/>
       <c r="K22" s="238"/>
     </row>
     <row r="23" spans="2:11" ht="15" customHeight="1">
-      <c r="B23" s="324" t="s">
+      <c r="B23" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C23" s="279"/>
@@ -6546,7 +6548,7 @@
       <c r="I23" s="258"/>
     </row>
     <row r="24" spans="2:11" ht="15" customHeight="1">
-      <c r="B24" s="333" t="s">
+      <c r="B24" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C24" s="279"/>
@@ -6557,14 +6559,14 @@
       <c r="F24" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G24" s="325" t="s">
+      <c r="G24" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H24" s="279"/>
       <c r="I24" s="213"/>
     </row>
     <row r="25" spans="2:11" ht="15" customHeight="1">
-      <c r="B25" s="322" t="s">
+      <c r="B25" s="321" t="s">
         <v>106</v>
       </c>
       <c r="C25" s="279"/>
@@ -6577,7 +6579,7 @@
         <f>E25/E19</f>
         <v>0.17142857142857143</v>
       </c>
-      <c r="G25" s="323">
+      <c r="G25" s="322">
         <v>1</v>
       </c>
       <c r="H25" s="279"/>
@@ -6597,14 +6599,14 @@
         <f>E26/E19</f>
         <v>0.47857142857142859</v>
       </c>
-      <c r="G26" s="323">
+      <c r="G26" s="322">
         <v>0.8</v>
       </c>
       <c r="H26" s="279"/>
       <c r="I26" s="213"/>
     </row>
     <row r="27" spans="2:11" ht="15" customHeight="1">
-      <c r="B27" s="347" t="s">
+      <c r="B27" s="348" t="s">
         <v>107</v>
       </c>
       <c r="C27" s="279"/>
@@ -6617,14 +6619,14 @@
         <f>E27/E19</f>
         <v>0.35</v>
       </c>
-      <c r="G27" s="323">
+      <c r="G27" s="322">
         <v>0.6</v>
       </c>
       <c r="H27" s="279"/>
       <c r="I27" s="213"/>
     </row>
     <row r="28" spans="2:11" ht="15" customHeight="1">
-      <c r="B28" s="319" t="s">
+      <c r="B28" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C28" s="246"/>
@@ -6637,7 +6639,7 @@
         <f>SUM(F25:F27)</f>
         <v>1</v>
       </c>
-      <c r="G28" s="310">
+      <c r="G28" s="309">
         <f>F25*G25+F26*G26+F27*G27</f>
         <v>0.76428571428571423</v>
       </c>
@@ -6655,7 +6657,7 @@
       <c r="I29" s="217"/>
     </row>
     <row r="30" spans="2:11" ht="15" customHeight="1">
-      <c r="B30" s="328" t="s">
+      <c r="B30" s="327" t="s">
         <v>118</v>
       </c>
       <c r="C30" s="279"/>
@@ -6667,19 +6669,19 @@
       <c r="I30" s="279"/>
     </row>
     <row r="31" spans="2:11" ht="15" customHeight="1">
-      <c r="B31" s="320" t="s">
+      <c r="B31" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C31" s="321"/>
-      <c r="D31" s="321"/>
-      <c r="E31" s="312" t="s">
+      <c r="C31" s="320"/>
+      <c r="D31" s="320"/>
+      <c r="E31" s="311" t="s">
         <v>119</v>
       </c>
       <c r="F31" s="279"/>
       <c r="G31" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H31" s="342" t="s">
+      <c r="H31" s="341" t="s">
         <v>120</v>
       </c>
       <c r="I31" s="258"/>
@@ -6689,38 +6691,38 @@
       </c>
     </row>
     <row r="32" spans="2:11" ht="15" customHeight="1">
-      <c r="B32" s="318" t="s">
+      <c r="B32" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C32" s="279"/>
       <c r="D32" s="279"/>
-      <c r="E32" s="335" t="s">
+      <c r="E32" s="334" t="s">
         <v>90</v>
       </c>
       <c r="F32" s="279"/>
       <c r="G32" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H32" s="345" t="s">
+      <c r="H32" s="344" t="s">
         <v>44</v>
       </c>
       <c r="I32" s="258"/>
       <c r="K32" s="203"/>
     </row>
     <row r="33" spans="2:11" ht="15" customHeight="1">
-      <c r="B33" s="318" t="s">
+      <c r="B33" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C33" s="279"/>
       <c r="D33" s="279"/>
-      <c r="E33" s="343">
+      <c r="E33" s="342">
         <v>1258.4000000000001</v>
       </c>
       <c r="F33" s="279"/>
       <c r="G33" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H33" s="345" t="s">
+      <c r="H33" s="344" t="s">
         <v>95</v>
       </c>
       <c r="I33" s="258"/>
@@ -6728,18 +6730,18 @@
     </row>
     <row r="34" spans="2:11" ht="15" customHeight="1">
       <c r="B34" s="211"/>
-      <c r="C34" s="334" t="s">
+      <c r="C34" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D34" s="279"/>
-      <c r="E34" s="340">
+      <c r="E34" s="339">
         <v>16900000</v>
       </c>
       <c r="F34" s="279"/>
       <c r="G34" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H34" s="316">
+      <c r="H34" s="315">
         <f>E34/E33</f>
         <v>13429.752066115701</v>
       </c>
@@ -6751,41 +6753,41 @@
     </row>
     <row r="35" spans="2:11" ht="15" customHeight="1">
       <c r="B35" s="212"/>
-      <c r="C35" s="334" t="s">
+      <c r="C35" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D35" s="279"/>
-      <c r="E35" s="356" t="s">
+      <c r="E35" s="355" t="s">
         <v>116</v>
       </c>
       <c r="F35" s="279"/>
       <c r="G35" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H35" s="317">
+      <c r="H35" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I35" s="258"/>
     </row>
     <row r="36" spans="2:11" ht="15" customHeight="1">
       <c r="B36" s="212"/>
-      <c r="C36" s="334" t="s">
+      <c r="C36" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D36" s="279"/>
-      <c r="E36" s="312" t="s">
+      <c r="E36" s="311" t="s">
         <v>97</v>
       </c>
       <c r="F36" s="279"/>
       <c r="G36" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H36" s="348"/>
+      <c r="H36" s="346"/>
       <c r="I36" s="258"/>
     </row>
     <row r="37" spans="2:11" ht="15" customHeight="1">
-      <c r="B37" s="324" t="s">
+      <c r="B37" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C37" s="279"/>
@@ -6798,7 +6800,7 @@
       <c r="K37" s="238"/>
     </row>
     <row r="38" spans="2:11" ht="15" customHeight="1">
-      <c r="B38" s="333" t="s">
+      <c r="B38" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C38" s="279"/>
@@ -6809,14 +6811,14 @@
       <c r="F38" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G38" s="325" t="s">
+      <c r="G38" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H38" s="279"/>
       <c r="I38" s="213"/>
     </row>
     <row r="39" spans="2:11" ht="15" customHeight="1">
-      <c r="B39" s="322" t="s">
+      <c r="B39" s="321" t="s">
         <v>106</v>
       </c>
       <c r="C39" s="279"/>
@@ -6828,7 +6830,7 @@
         <f>E39/E33</f>
         <v>0.11538461538461536</v>
       </c>
-      <c r="G39" s="323">
+      <c r="G39" s="322">
         <v>1</v>
       </c>
       <c r="H39" s="279"/>
@@ -6848,14 +6850,14 @@
         <f>E40/E33</f>
         <v>0.53341538461538451</v>
       </c>
-      <c r="G40" s="323">
+      <c r="G40" s="322">
         <v>0.8</v>
       </c>
       <c r="H40" s="279"/>
       <c r="I40" s="213"/>
     </row>
     <row r="41" spans="2:11" ht="15" customHeight="1">
-      <c r="B41" s="347" t="s">
+      <c r="B41" s="348" t="s">
         <v>107</v>
       </c>
       <c r="C41" s="279"/>
@@ -6868,14 +6870,14 @@
         <f>E41/E33</f>
         <v>0.35120000000000001</v>
       </c>
-      <c r="G41" s="323">
+      <c r="G41" s="322">
         <v>0.6</v>
       </c>
       <c r="H41" s="279"/>
       <c r="I41" s="213"/>
     </row>
     <row r="42" spans="2:11" ht="15" customHeight="1">
-      <c r="B42" s="319" t="s">
+      <c r="B42" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C42" s="246"/>
@@ -6888,7 +6890,7 @@
         <f>F39+F41+F40</f>
         <v>0.99999999999999989</v>
       </c>
-      <c r="G42" s="310">
+      <c r="G42" s="309">
         <f>F41*G41+F39*G39+F40*G40</f>
         <v>0.75283692307692296</v>
       </c>
@@ -6906,7 +6908,7 @@
       <c r="I43" s="173"/>
     </row>
     <row r="44" spans="2:11" ht="15" customHeight="1">
-      <c r="B44" s="344" t="s">
+      <c r="B44" s="343" t="s">
         <v>122</v>
       </c>
       <c r="C44" s="279"/>
@@ -6918,19 +6920,19 @@
       <c r="I44" s="279"/>
     </row>
     <row r="45" spans="2:11" ht="15" customHeight="1">
-      <c r="B45" s="320" t="s">
+      <c r="B45" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C45" s="321"/>
-      <c r="D45" s="321"/>
-      <c r="E45" s="335" t="s">
+      <c r="C45" s="320"/>
+      <c r="D45" s="320"/>
+      <c r="E45" s="334" t="s">
         <v>119</v>
       </c>
       <c r="F45" s="279"/>
       <c r="G45" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H45" s="342" t="s">
+      <c r="H45" s="341" t="s">
         <v>120</v>
       </c>
       <c r="I45" s="258"/>
@@ -6939,37 +6941,37 @@
       </c>
     </row>
     <row r="46" spans="2:11" ht="15" customHeight="1">
-      <c r="B46" s="318" t="s">
+      <c r="B46" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C46" s="279"/>
       <c r="D46" s="279"/>
-      <c r="E46" s="335" t="s">
+      <c r="E46" s="334" t="s">
         <v>90</v>
       </c>
       <c r="F46" s="279"/>
       <c r="G46" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H46" s="345" t="s">
+      <c r="H46" s="344" t="s">
         <v>49</v>
       </c>
       <c r="I46" s="258"/>
     </row>
     <row r="47" spans="2:11" ht="15" customHeight="1">
-      <c r="B47" s="318" t="s">
+      <c r="B47" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C47" s="279"/>
       <c r="D47" s="279"/>
-      <c r="E47" s="352">
+      <c r="E47" s="351">
         <v>430.76</v>
       </c>
       <c r="F47" s="279"/>
       <c r="G47" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H47" s="315" t="s">
+      <c r="H47" s="314" t="s">
         <v>95</v>
       </c>
       <c r="I47" s="258"/>
@@ -6977,18 +6979,18 @@
     </row>
     <row r="48" spans="2:11" ht="15" customHeight="1">
       <c r="B48" s="164"/>
-      <c r="C48" s="334" t="s">
+      <c r="C48" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D48" s="279"/>
-      <c r="E48" s="311">
+      <c r="E48" s="310">
         <v>7120000</v>
       </c>
       <c r="F48" s="279"/>
       <c r="G48" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H48" s="331">
+      <c r="H48" s="330">
         <f>E48/E47</f>
         <v>16528.92561983471</v>
       </c>
@@ -7001,42 +7003,42 @@
     </row>
     <row r="49" spans="2:11" ht="15" customHeight="1">
       <c r="B49" s="165"/>
-      <c r="C49" s="334" t="s">
+      <c r="C49" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D49" s="279"/>
-      <c r="E49" s="356" t="s">
+      <c r="E49" s="355" t="s">
         <v>116</v>
       </c>
       <c r="F49" s="279"/>
       <c r="G49" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H49" s="317">
+      <c r="H49" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I49" s="258"/>
     </row>
     <row r="50" spans="2:11" ht="15" customHeight="1">
       <c r="B50" s="165"/>
-      <c r="C50" s="334" t="s">
+      <c r="C50" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D50" s="279"/>
-      <c r="E50" s="312" t="s">
+      <c r="E50" s="311" t="s">
         <v>124</v>
       </c>
       <c r="F50" s="279"/>
       <c r="G50" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H50" s="336"/>
+      <c r="H50" s="335"/>
       <c r="I50" s="258"/>
       <c r="K50" s="238"/>
     </row>
     <row r="51" spans="2:11" ht="15" customHeight="1">
-      <c r="B51" s="324" t="s">
+      <c r="B51" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C51" s="279"/>
@@ -7048,7 +7050,7 @@
       <c r="I51" s="258"/>
     </row>
     <row r="52" spans="2:11" ht="15" customHeight="1">
-      <c r="B52" s="333" t="s">
+      <c r="B52" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C52" s="279"/>
@@ -7059,14 +7061,14 @@
       <c r="F52" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G52" s="325" t="s">
+      <c r="G52" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H52" s="279"/>
       <c r="I52" s="167"/>
     </row>
     <row r="53" spans="2:11" ht="15" customHeight="1">
-      <c r="B53" s="322" t="s">
+      <c r="B53" s="321" t="s">
         <v>106</v>
       </c>
       <c r="C53" s="279"/>
@@ -7078,7 +7080,7 @@
         <f>E53/E47</f>
         <v>0.33707865168539325</v>
       </c>
-      <c r="G53" s="314">
+      <c r="G53" s="313">
         <v>1</v>
       </c>
       <c r="H53" s="279"/>
@@ -7098,7 +7100,7 @@
         <f>E54/E47</f>
         <v>0.31042134831460677</v>
       </c>
-      <c r="G54" s="314">
+      <c r="G54" s="313">
         <v>0.8</v>
       </c>
       <c r="H54" s="279"/>
@@ -7118,14 +7120,14 @@
         <f>E55/E47</f>
         <v>0.35249999999999998</v>
       </c>
-      <c r="G55" s="314">
+      <c r="G55" s="313">
         <v>0.6</v>
       </c>
       <c r="H55" s="279"/>
       <c r="I55" s="167"/>
     </row>
     <row r="56" spans="2:11" ht="15" customHeight="1">
-      <c r="B56" s="319" t="s">
+      <c r="B56" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C56" s="246"/>
@@ -7138,7 +7140,7 @@
         <f>SUM(F53:F55)</f>
         <v>1</v>
       </c>
-      <c r="G56" s="310">
+      <c r="G56" s="309">
         <f>F53*G53+F55*G55+F54*G54</f>
         <v>0.79691573033707863</v>
       </c>
@@ -7156,7 +7158,7 @@
       <c r="I57" s="173"/>
     </row>
     <row r="58" spans="2:11" ht="15" customHeight="1">
-      <c r="B58" s="328" t="s">
+      <c r="B58" s="327" t="s">
         <v>125</v>
       </c>
       <c r="C58" s="279"/>
@@ -7169,19 +7171,19 @@
       <c r="K58" s="203"/>
     </row>
     <row r="59" spans="2:11" ht="15" customHeight="1">
-      <c r="B59" s="320" t="s">
+      <c r="B59" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C59" s="321"/>
-      <c r="D59" s="321"/>
-      <c r="E59" s="335" t="s">
+      <c r="C59" s="320"/>
+      <c r="D59" s="320"/>
+      <c r="E59" s="334" t="s">
         <v>126</v>
       </c>
       <c r="F59" s="279"/>
       <c r="G59" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H59" s="355" t="s">
+      <c r="H59" s="354" t="s">
         <v>127</v>
       </c>
       <c r="I59" s="258"/>
@@ -7190,55 +7192,55 @@
       </c>
     </row>
     <row r="60" spans="2:11" ht="15" customHeight="1">
-      <c r="B60" s="318" t="s">
+      <c r="B60" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C60" s="279"/>
       <c r="D60" s="279"/>
-      <c r="E60" s="335" t="s">
+      <c r="E60" s="334" t="s">
         <v>90</v>
       </c>
       <c r="F60" s="279"/>
       <c r="G60" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H60" s="345" t="s">
+      <c r="H60" s="344" t="s">
         <v>49</v>
       </c>
       <c r="I60" s="258"/>
     </row>
     <row r="61" spans="2:11" ht="15" customHeight="1">
-      <c r="B61" s="318" t="s">
+      <c r="B61" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C61" s="279"/>
       <c r="D61" s="279"/>
-      <c r="E61" s="326">
+      <c r="E61" s="325">
         <v>626</v>
       </c>
       <c r="F61" s="279"/>
       <c r="G61" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H61" s="345" t="s">
+      <c r="H61" s="344" t="s">
         <v>129</v>
       </c>
       <c r="I61" s="258"/>
     </row>
     <row r="62" spans="2:11" ht="15" customHeight="1">
       <c r="B62" s="164"/>
-      <c r="C62" s="334" t="s">
+      <c r="C62" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D62" s="279"/>
-      <c r="E62" s="350">
+      <c r="E62" s="349">
         <v>10500000</v>
       </c>
       <c r="F62" s="279"/>
       <c r="G62" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H62" s="327">
+      <c r="H62" s="326">
         <f>E62/E61</f>
         <v>16773.162939297126</v>
       </c>
@@ -7251,42 +7253,42 @@
     </row>
     <row r="63" spans="2:11" ht="15" customHeight="1">
       <c r="B63" s="165"/>
-      <c r="C63" s="334" t="s">
+      <c r="C63" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D63" s="279"/>
-      <c r="E63" s="349" t="s">
+      <c r="E63" s="347" t="s">
         <v>116</v>
       </c>
       <c r="F63" s="279"/>
       <c r="G63" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H63" s="317">
+      <c r="H63" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I63" s="258"/>
     </row>
     <row r="64" spans="2:11" ht="15" customHeight="1">
       <c r="B64" s="165"/>
-      <c r="C64" s="334" t="s">
+      <c r="C64" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D64" s="279"/>
-      <c r="E64" s="312" t="s">
+      <c r="E64" s="311" t="s">
         <v>97</v>
       </c>
       <c r="F64" s="279"/>
       <c r="G64" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H64" s="336"/>
+      <c r="H64" s="335"/>
       <c r="I64" s="258"/>
       <c r="K64" s="238"/>
     </row>
     <row r="65" spans="2:11" ht="15" customHeight="1">
-      <c r="B65" s="324" t="s">
+      <c r="B65" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C65" s="279"/>
@@ -7298,7 +7300,7 @@
       <c r="I65" s="258"/>
     </row>
     <row r="66" spans="2:11" ht="15" customHeight="1">
-      <c r="B66" s="333" t="s">
+      <c r="B66" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C66" s="279"/>
@@ -7309,7 +7311,7 @@
       <c r="F66" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G66" s="325" t="s">
+      <c r="G66" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H66" s="279"/>
@@ -7328,7 +7330,7 @@
         <f>E67/E61</f>
         <v>0.30830670926517573</v>
       </c>
-      <c r="G67" s="314">
+      <c r="G67" s="313">
         <v>1</v>
       </c>
       <c r="H67" s="279"/>
@@ -7347,14 +7349,14 @@
         <f>E68/E61</f>
         <v>0.27156549520766771</v>
       </c>
-      <c r="G68" s="314">
+      <c r="G68" s="313">
         <v>0.9</v>
       </c>
       <c r="H68" s="279"/>
       <c r="I68" s="167"/>
     </row>
     <row r="69" spans="2:11" ht="15" customHeight="1">
-      <c r="B69" s="358" t="s">
+      <c r="B69" s="350" t="s">
         <v>107</v>
       </c>
       <c r="C69" s="279"/>
@@ -7367,14 +7369,14 @@
         <f>E69/E61</f>
         <v>0.42012779552715657</v>
       </c>
-      <c r="G69" s="314">
+      <c r="G69" s="313">
         <v>0.6</v>
       </c>
       <c r="H69" s="279"/>
       <c r="I69" s="167"/>
     </row>
     <row r="70" spans="2:11" ht="15" customHeight="1">
-      <c r="B70" s="319" t="s">
+      <c r="B70" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C70" s="246"/>
@@ -7387,7 +7389,7 @@
         <f>SUM(F67:F69)</f>
         <v>1</v>
       </c>
-      <c r="G70" s="310">
+      <c r="G70" s="309">
         <f>F67*G67+F69*G69+F68*G68</f>
         <v>0.80479233226837055</v>
       </c>
@@ -7405,7 +7407,7 @@
       <c r="I71" s="173"/>
     </row>
     <row r="72" spans="2:11" ht="15" customHeight="1">
-      <c r="B72" s="328" t="s">
+      <c r="B72" s="327" t="s">
         <v>131</v>
       </c>
       <c r="C72" s="279"/>
@@ -7417,19 +7419,19 @@
       <c r="I72" s="279"/>
     </row>
     <row r="73" spans="2:11" ht="15" customHeight="1">
-      <c r="B73" s="320" t="s">
+      <c r="B73" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C73" s="321"/>
-      <c r="D73" s="321"/>
-      <c r="E73" s="312" t="s">
+      <c r="C73" s="320"/>
+      <c r="D73" s="320"/>
+      <c r="E73" s="311" t="s">
         <v>132</v>
       </c>
       <c r="F73" s="279"/>
       <c r="G73" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H73" s="342" t="s">
+      <c r="H73" s="341" t="s">
         <v>133</v>
       </c>
       <c r="I73" s="258"/>
@@ -7438,30 +7440,30 @@
       </c>
     </row>
     <row r="74" spans="2:11" ht="15" customHeight="1">
-      <c r="B74" s="318" t="s">
+      <c r="B74" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C74" s="279"/>
       <c r="D74" s="279"/>
-      <c r="E74" s="312" t="s">
+      <c r="E74" s="311" t="s">
         <v>135</v>
       </c>
       <c r="F74" s="279"/>
       <c r="G74" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H74" s="345" t="s">
+      <c r="H74" s="344" t="s">
         <v>49</v>
       </c>
       <c r="I74" s="258"/>
     </row>
     <row r="75" spans="2:11" ht="15" customHeight="1">
-      <c r="B75" s="318" t="s">
+      <c r="B75" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C75" s="279"/>
       <c r="D75" s="279"/>
-      <c r="E75" s="329">
+      <c r="E75" s="328">
         <f>730 *4.84</f>
         <v>3533.2</v>
       </c>
@@ -7469,25 +7471,25 @@
       <c r="G75" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H75" s="315" t="s">
+      <c r="H75" s="314" t="s">
         <v>95</v>
       </c>
       <c r="I75" s="258"/>
     </row>
     <row r="76" spans="2:11" ht="15" customHeight="1">
       <c r="B76" s="164"/>
-      <c r="C76" s="334" t="s">
+      <c r="C76" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D76" s="279"/>
-      <c r="E76" s="311">
+      <c r="E76" s="310">
         <v>60000000</v>
       </c>
       <c r="F76" s="279"/>
       <c r="G76" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H76" s="331">
+      <c r="H76" s="330">
         <f>E76/E75</f>
         <v>16981.772897090457</v>
       </c>
@@ -7495,20 +7497,20 @@
     </row>
     <row r="77" spans="2:11" ht="15" customHeight="1">
       <c r="B77" s="165"/>
-      <c r="C77" s="334" t="s">
+      <c r="C77" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D77" s="279"/>
-      <c r="E77" s="364" t="s">
+      <c r="E77" s="363" t="s">
         <v>116</v>
       </c>
       <c r="F77" s="279"/>
       <c r="G77" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H77" s="317">
+      <c r="H77" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I77" s="258"/>
       <c r="K77" s="221">
@@ -7518,22 +7520,22 @@
     </row>
     <row r="78" spans="2:11" ht="15" customHeight="1">
       <c r="B78" s="165"/>
-      <c r="C78" s="334" t="s">
+      <c r="C78" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D78" s="279"/>
-      <c r="E78" s="312" t="s">
+      <c r="E78" s="311" t="s">
         <v>136</v>
       </c>
       <c r="F78" s="279"/>
       <c r="G78" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H78" s="336"/>
+      <c r="H78" s="335"/>
       <c r="I78" s="258"/>
     </row>
     <row r="79" spans="2:11" ht="15" customHeight="1">
-      <c r="B79" s="324" t="s">
+      <c r="B79" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C79" s="279"/>
@@ -7546,7 +7548,7 @@
       <c r="K79" s="238"/>
     </row>
     <row r="80" spans="2:11" ht="15" customHeight="1">
-      <c r="B80" s="333" t="s">
+      <c r="B80" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C80" s="279"/>
@@ -7557,14 +7559,14 @@
       <c r="F80" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G80" s="325" t="s">
+      <c r="G80" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H80" s="279"/>
       <c r="I80" s="167"/>
     </row>
     <row r="81" spans="2:11" ht="15" customHeight="1">
-      <c r="B81" s="332" t="s">
+      <c r="B81" s="331" t="s">
         <v>130</v>
       </c>
       <c r="C81" s="279"/>
@@ -7577,14 +7579,14 @@
         <f>E81/E75</f>
         <v>0.56164383561643838</v>
       </c>
-      <c r="G81" s="314">
+      <c r="G81" s="313">
         <v>0.9</v>
       </c>
       <c r="H81" s="279"/>
       <c r="I81" s="167"/>
     </row>
     <row r="82" spans="2:11" ht="15" customHeight="1">
-      <c r="B82" s="332" t="s">
+      <c r="B82" s="331" t="s">
         <v>117</v>
       </c>
       <c r="C82" s="279"/>
@@ -7597,7 +7599,7 @@
         <f>E82/E75</f>
         <v>8.6756164383561624E-2</v>
       </c>
-      <c r="G82" s="314">
+      <c r="G82" s="313">
         <v>0.8</v>
       </c>
       <c r="H82" s="279"/>
@@ -7617,14 +7619,14 @@
         <f>E83/E75</f>
         <v>0.35160000000000002</v>
       </c>
-      <c r="G83" s="314">
+      <c r="G83" s="313">
         <v>0.6</v>
       </c>
       <c r="H83" s="279"/>
       <c r="I83" s="167"/>
     </row>
     <row r="84" spans="2:11" ht="15" customHeight="1">
-      <c r="B84" s="319" t="s">
+      <c r="B84" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C84" s="246"/>
@@ -7637,7 +7639,7 @@
         <f>SUM(F81:F83)</f>
         <v>1</v>
       </c>
-      <c r="G84" s="310">
+      <c r="G84" s="309">
         <f>F81*G81+F83*G83+F82*G82</f>
         <v>0.78584438356164399</v>
       </c>
@@ -7655,7 +7657,7 @@
       <c r="I85" s="173"/>
     </row>
     <row r="86" spans="2:11" ht="15" customHeight="1">
-      <c r="B86" s="328" t="s">
+      <c r="B86" s="327" t="s">
         <v>137</v>
       </c>
       <c r="C86" s="279"/>
@@ -7668,19 +7670,19 @@
       <c r="K86" s="203"/>
     </row>
     <row r="87" spans="2:11" ht="15" customHeight="1">
-      <c r="B87" s="320" t="s">
+      <c r="B87" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C87" s="321"/>
-      <c r="D87" s="321"/>
-      <c r="E87" s="335" t="s">
+      <c r="C87" s="320"/>
+      <c r="D87" s="320"/>
+      <c r="E87" s="334" t="s">
         <v>119</v>
       </c>
       <c r="F87" s="279"/>
       <c r="G87" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H87" s="357" t="str">
+      <c r="H87" s="356" t="str">
         <f>H45</f>
         <v>(63) 99252-2282</v>
       </c>
@@ -7690,30 +7692,30 @@
       </c>
     </row>
     <row r="88" spans="2:11" ht="15" customHeight="1">
-      <c r="B88" s="318" t="s">
+      <c r="B88" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C88" s="279"/>
       <c r="D88" s="279"/>
-      <c r="E88" s="335" t="s">
+      <c r="E88" s="334" t="s">
         <v>90</v>
       </c>
       <c r="F88" s="279"/>
       <c r="G88" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H88" s="345" t="s">
+      <c r="H88" s="344" t="s">
         <v>49</v>
       </c>
       <c r="I88" s="258"/>
     </row>
     <row r="89" spans="2:11" ht="15" customHeight="1">
-      <c r="B89" s="318" t="s">
+      <c r="B89" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C89" s="279"/>
       <c r="D89" s="279"/>
-      <c r="E89" s="343">
+      <c r="E89" s="342">
         <f>733*4.84</f>
         <v>3547.72</v>
       </c>
@@ -7721,25 +7723,25 @@
       <c r="G89" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H89" s="315" t="s">
+      <c r="H89" s="314" t="s">
         <v>95</v>
       </c>
       <c r="I89" s="258"/>
     </row>
     <row r="90" spans="2:11" ht="15" customHeight="1">
       <c r="B90" s="164"/>
-      <c r="C90" s="334" t="s">
+      <c r="C90" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D90" s="279"/>
-      <c r="E90" s="337">
+      <c r="E90" s="336">
         <v>43980000</v>
       </c>
       <c r="F90" s="279"/>
       <c r="G90" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H90" s="327">
+      <c r="H90" s="326">
         <f>E90/E89</f>
         <v>12396.694214876034</v>
       </c>
@@ -7751,41 +7753,41 @@
     </row>
     <row r="91" spans="2:11" ht="15" customHeight="1">
       <c r="B91" s="165"/>
-      <c r="C91" s="334" t="s">
+      <c r="C91" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D91" s="279"/>
-      <c r="E91" s="362" t="s">
+      <c r="E91" s="361" t="s">
         <v>116</v>
       </c>
       <c r="F91" s="279"/>
       <c r="G91" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H91" s="317">
+      <c r="H91" s="316">
         <f ca="1">TODAY()</f>
-        <v>45824</v>
+        <v>45828</v>
       </c>
       <c r="I91" s="258"/>
     </row>
     <row r="92" spans="2:11" ht="15" customHeight="1">
       <c r="B92" s="165"/>
-      <c r="C92" s="334" t="s">
+      <c r="C92" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D92" s="279"/>
-      <c r="E92" s="312" t="s">
+      <c r="E92" s="311" t="s">
         <v>97</v>
       </c>
       <c r="F92" s="279"/>
       <c r="G92" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H92" s="336"/>
+      <c r="H92" s="335"/>
       <c r="I92" s="258"/>
     </row>
     <row r="93" spans="2:11" ht="15" customHeight="1">
-      <c r="B93" s="324" t="s">
+      <c r="B93" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C93" s="279"/>
@@ -7797,7 +7799,7 @@
       <c r="I93" s="258"/>
     </row>
     <row r="94" spans="2:11" ht="15" customHeight="1">
-      <c r="B94" s="333" t="s">
+      <c r="B94" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C94" s="279"/>
@@ -7808,14 +7810,14 @@
       <c r="F94" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G94" s="325" t="s">
+      <c r="G94" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H94" s="279"/>
       <c r="I94" s="167"/>
     </row>
     <row r="95" spans="2:11" ht="15" customHeight="1">
-      <c r="B95" s="322" t="s">
+      <c r="B95" s="321" t="s">
         <v>106</v>
       </c>
       <c r="C95" s="279"/>
@@ -7827,7 +7829,7 @@
         <f>E95/E89</f>
         <v>0.31005829095870024</v>
       </c>
-      <c r="G95" s="366">
+      <c r="G95" s="365">
         <v>1</v>
       </c>
       <c r="H95" s="279"/>
@@ -7847,14 +7849,14 @@
         <f>E96/E89</f>
         <v>0.33854170904129977</v>
       </c>
-      <c r="G96" s="366">
+      <c r="G96" s="365">
         <v>0.8</v>
       </c>
       <c r="H96" s="279"/>
       <c r="I96" s="206"/>
     </row>
     <row r="97" spans="2:12" ht="15" customHeight="1">
-      <c r="B97" s="363" t="s">
+      <c r="B97" s="362" t="s">
         <v>107</v>
       </c>
       <c r="C97" s="279"/>
@@ -7867,7 +7869,7 @@
         <f>E97/E89</f>
         <v>0.35139999999999999</v>
       </c>
-      <c r="G97" s="314">
+      <c r="G97" s="313">
         <v>0.6</v>
       </c>
       <c r="H97" s="279"/>
@@ -7876,7 +7878,7 @@
       <c r="L97" s="207"/>
     </row>
     <row r="98" spans="2:12" ht="15" customHeight="1">
-      <c r="B98" s="319" t="s">
+      <c r="B98" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C98" s="246"/>
@@ -7889,7 +7891,7 @@
         <f>SUM(F95:F97)</f>
         <v>1</v>
       </c>
-      <c r="G98" s="310">
+      <c r="G98" s="309">
         <f>F97*G97+F95*G95+F96*G96</f>
         <v>0.79173165819173996</v>
       </c>
@@ -7914,7 +7916,7 @@
       <c r="L99" s="207"/>
     </row>
     <row r="100" spans="2:12" ht="15" customHeight="1">
-      <c r="B100" s="330"/>
+      <c r="B100" s="329"/>
       <c r="C100" s="279"/>
       <c r="D100" s="279"/>
       <c r="E100" s="279"/>
@@ -7926,7 +7928,7 @@
       <c r="L100" s="207"/>
     </row>
     <row r="101" spans="2:12" ht="15" customHeight="1">
-      <c r="B101" s="328" t="s">
+      <c r="B101" s="327" t="s">
         <v>139</v>
       </c>
       <c r="C101" s="279"/>
@@ -7940,93 +7942,93 @@
       <c r="L101" s="207"/>
     </row>
     <row r="102" spans="2:12" ht="15" customHeight="1">
-      <c r="B102" s="320" t="s">
+      <c r="B102" s="319" t="s">
         <v>109</v>
       </c>
-      <c r="C102" s="321"/>
-      <c r="D102" s="321"/>
-      <c r="E102" s="372"/>
+      <c r="C102" s="320"/>
+      <c r="D102" s="320"/>
+      <c r="E102" s="371"/>
       <c r="F102" s="279"/>
       <c r="G102" s="163" t="s">
         <v>87</v>
       </c>
-      <c r="H102" s="313"/>
+      <c r="H102" s="312"/>
       <c r="I102" s="258"/>
       <c r="K102" s="207"/>
       <c r="L102" s="207"/>
     </row>
     <row r="103" spans="2:12" ht="15" customHeight="1">
-      <c r="B103" s="318" t="s">
+      <c r="B103" s="317" t="s">
         <v>89</v>
       </c>
       <c r="C103" s="279"/>
       <c r="D103" s="279"/>
-      <c r="E103" s="367"/>
+      <c r="E103" s="366"/>
       <c r="F103" s="279"/>
       <c r="G103" s="163" t="s">
         <v>91</v>
       </c>
-      <c r="H103" s="361"/>
+      <c r="H103" s="360"/>
       <c r="I103" s="258"/>
     </row>
     <row r="104" spans="2:12" ht="15" customHeight="1">
-      <c r="B104" s="318" t="s">
+      <c r="B104" s="317" t="s">
         <v>93</v>
       </c>
       <c r="C104" s="279"/>
       <c r="D104" s="279"/>
-      <c r="E104" s="326"/>
+      <c r="E104" s="325"/>
       <c r="F104" s="279"/>
       <c r="G104" s="163" t="s">
         <v>94</v>
       </c>
-      <c r="H104" s="339"/>
+      <c r="H104" s="338"/>
       <c r="I104" s="258"/>
     </row>
     <row r="105" spans="2:12" ht="15" customHeight="1">
       <c r="B105" s="164"/>
-      <c r="C105" s="334" t="s">
+      <c r="C105" s="333" t="s">
         <v>113</v>
       </c>
       <c r="D105" s="279"/>
-      <c r="E105" s="337"/>
+      <c r="E105" s="336"/>
       <c r="F105" s="279"/>
       <c r="G105" s="163" t="s">
         <v>114</v>
       </c>
-      <c r="H105" s="327"/>
+      <c r="H105" s="326"/>
       <c r="I105" s="258"/>
     </row>
     <row r="106" spans="2:12" ht="15" customHeight="1">
       <c r="B106" s="165"/>
-      <c r="C106" s="334" t="s">
+      <c r="C106" s="333" t="s">
         <v>115</v>
       </c>
       <c r="D106" s="279"/>
-      <c r="E106" s="362"/>
+      <c r="E106" s="361"/>
       <c r="F106" s="279"/>
       <c r="G106" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="H106" s="365"/>
+      <c r="H106" s="364"/>
       <c r="I106" s="258"/>
     </row>
     <row r="107" spans="2:12" ht="15" customHeight="1">
       <c r="B107" s="165"/>
-      <c r="C107" s="334" t="s">
+      <c r="C107" s="333" t="s">
         <v>96</v>
       </c>
       <c r="D107" s="279"/>
-      <c r="E107" s="338"/>
+      <c r="E107" s="337"/>
       <c r="F107" s="279"/>
       <c r="G107" s="163" t="s">
         <v>100</v>
       </c>
-      <c r="H107" s="336"/>
+      <c r="H107" s="335"/>
       <c r="I107" s="258"/>
     </row>
     <row r="108" spans="2:12" ht="15" customHeight="1">
-      <c r="B108" s="324" t="s">
+      <c r="B108" s="323" t="s">
         <v>101</v>
       </c>
       <c r="C108" s="279"/>
@@ -8038,7 +8040,7 @@
       <c r="I108" s="258"/>
     </row>
     <row r="109" spans="2:12" ht="15" customHeight="1">
-      <c r="B109" s="333" t="s">
+      <c r="B109" s="332" t="s">
         <v>102</v>
       </c>
       <c r="C109" s="279"/>
@@ -8049,38 +8051,38 @@
       <c r="F109" s="166" t="s">
         <v>104</v>
       </c>
-      <c r="G109" s="325" t="s">
+      <c r="G109" s="324" t="s">
         <v>105</v>
       </c>
       <c r="H109" s="279"/>
       <c r="I109" s="167"/>
     </row>
     <row r="110" spans="2:12" ht="15" customHeight="1">
-      <c r="B110" s="363" t="s">
+      <c r="B110" s="362" t="s">
         <v>106</v>
       </c>
       <c r="C110" s="279"/>
       <c r="D110" s="279"/>
       <c r="E110" s="168"/>
       <c r="F110" s="169"/>
-      <c r="G110" s="314"/>
+      <c r="G110" s="313"/>
       <c r="H110" s="279"/>
       <c r="I110" s="167"/>
     </row>
     <row r="111" spans="2:12" ht="15" customHeight="1">
-      <c r="B111" s="363" t="s">
+      <c r="B111" s="362" t="s">
         <v>107</v>
       </c>
       <c r="C111" s="279"/>
       <c r="D111" s="279"/>
       <c r="E111" s="168"/>
       <c r="F111" s="169"/>
-      <c r="G111" s="314"/>
+      <c r="G111" s="313"/>
       <c r="H111" s="279"/>
       <c r="I111" s="167"/>
     </row>
     <row r="112" spans="2:12" ht="15" customHeight="1">
-      <c r="B112" s="319" t="s">
+      <c r="B112" s="318" t="s">
         <v>83</v>
       </c>
       <c r="C112" s="246"/>
@@ -8093,7 +8095,7 @@
         <f>SUM(F110:F111)</f>
         <v>0</v>
       </c>
-      <c r="G112" s="310">
+      <c r="G112" s="309">
         <f>F110*G110+F111*G111</f>
         <v>0</v>
       </c>
@@ -8174,7 +8176,6 @@
     <mergeCell ref="E77:F77"/>
     <mergeCell ref="E50:F50"/>
     <mergeCell ref="H35:I35"/>
-    <mergeCell ref="H18:I18"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B79:I79"/>
     <mergeCell ref="G25:H25"/>
@@ -8194,6 +8195,10 @@
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="E59:F59"/>
     <mergeCell ref="B51:I51"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="H17:I17"/>
     <mergeCell ref="H107:I107"/>
     <mergeCell ref="C78:D78"/>
     <mergeCell ref="C35:D35"/>
@@ -8218,16 +8223,6 @@
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="G53:H53"/>
     <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="B42:D42"/>
-    <mergeCell ref="E78:F78"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="H49:I49"/>
-    <mergeCell ref="E74:F74"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="B16:I16"/>
     <mergeCell ref="E33:F33"/>
@@ -8239,12 +8234,11 @@
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C76:D76"/>
     <mergeCell ref="B66:D66"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="B17:D17"/>
-    <mergeCell ref="G82:H82"/>
+    <mergeCell ref="H18:I18"/>
     <mergeCell ref="H36:I36"/>
     <mergeCell ref="B61:D61"/>
     <mergeCell ref="C63:D63"/>
@@ -8254,18 +8248,21 @@
     <mergeCell ref="C77:D77"/>
     <mergeCell ref="E31:F31"/>
     <mergeCell ref="H33:I33"/>
-    <mergeCell ref="B80:D80"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="E46:F46"/>
-    <mergeCell ref="G81:H81"/>
     <mergeCell ref="C62:D62"/>
     <mergeCell ref="E62:F62"/>
     <mergeCell ref="C49:D49"/>
-    <mergeCell ref="G80:H80"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="B75:D75"/>
     <mergeCell ref="B69:D69"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="E74:F74"/>
+    <mergeCell ref="C76:D76"/>
     <mergeCell ref="E107:F107"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="B102:D102"/>
@@ -8307,6 +8304,11 @@
     <mergeCell ref="H78:I78"/>
     <mergeCell ref="E90:F90"/>
     <mergeCell ref="B84:D84"/>
+    <mergeCell ref="G82:H82"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="G81:H81"/>
+    <mergeCell ref="G80:H80"/>
+    <mergeCell ref="E78:F78"/>
     <mergeCell ref="G112:H112"/>
     <mergeCell ref="E48:F48"/>
     <mergeCell ref="E22:F22"/>
@@ -8682,16 +8684,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15" customHeight="1">
-      <c r="E1" s="375"/>
-      <c r="F1" s="376"/>
-      <c r="G1" s="376"/>
-      <c r="H1" s="376"/>
-      <c r="I1" s="376"/>
-      <c r="J1" s="376"/>
-      <c r="K1" s="376"/>
-      <c r="L1" s="376"/>
-      <c r="M1" s="376"/>
-      <c r="N1" s="376"/>
+      <c r="E1" s="374"/>
+      <c r="F1" s="375"/>
+      <c r="G1" s="375"/>
+      <c r="H1" s="375"/>
+      <c r="I1" s="375"/>
+      <c r="J1" s="375"/>
+      <c r="K1" s="375"/>
+      <c r="L1" s="375"/>
+      <c r="M1" s="375"/>
+      <c r="N1" s="375"/>
     </row>
     <row r="2" spans="1:18" ht="13.5" customHeight="1" thickBot="1"/>
     <row r="3" spans="1:18" ht="45" customHeight="1">
@@ -9239,21 +9241,21 @@
       <c r="R11" s="146"/>
     </row>
     <row r="12" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A12" s="374" t="s">
+      <c r="A12" s="373" t="s">
         <v>173</v>
       </c>
       <c r="B12" s="244"/>
-      <c r="C12" s="377" t="s">
+      <c r="C12" s="376" t="s">
         <v>174</v>
       </c>
-      <c r="D12" s="376"/>
-      <c r="E12" s="376"/>
-      <c r="F12" s="376"/>
-      <c r="G12" s="376"/>
-      <c r="H12" s="376"/>
-      <c r="I12" s="376"/>
-      <c r="J12" s="376"/>
-      <c r="K12" s="376"/>
+      <c r="D12" s="375"/>
+      <c r="E12" s="375"/>
+      <c r="F12" s="375"/>
+      <c r="G12" s="375"/>
+      <c r="H12" s="375"/>
+      <c r="I12" s="375"/>
+      <c r="J12" s="375"/>
+      <c r="K12" s="375"/>
       <c r="L12" s="145"/>
       <c r="M12" s="144"/>
       <c r="N12" s="144"/>
@@ -9268,21 +9270,21 @@
       <c r="R12" s="146"/>
     </row>
     <row r="13" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A13" s="374" t="s">
+      <c r="A13" s="373" t="s">
         <v>176</v>
       </c>
       <c r="B13" s="244"/>
-      <c r="C13" s="377" t="s">
+      <c r="C13" s="376" t="s">
         <v>177</v>
       </c>
-      <c r="D13" s="376"/>
-      <c r="E13" s="376"/>
-      <c r="F13" s="376"/>
-      <c r="G13" s="376"/>
-      <c r="H13" s="376"/>
-      <c r="I13" s="376"/>
-      <c r="J13" s="376"/>
-      <c r="K13" s="376"/>
+      <c r="D13" s="375"/>
+      <c r="E13" s="375"/>
+      <c r="F13" s="375"/>
+      <c r="G13" s="375"/>
+      <c r="H13" s="375"/>
+      <c r="I13" s="375"/>
+      <c r="J13" s="375"/>
+      <c r="K13" s="375"/>
       <c r="L13" s="144"/>
       <c r="M13" s="144"/>
       <c r="N13" s="144"/>
@@ -9297,22 +9299,22 @@
       <c r="R13" s="146"/>
     </row>
     <row r="14" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A14" s="374" t="str">
+      <c r="A14" s="373" t="str">
         <f>L3</f>
         <v>Benfeitorias Indexado³</v>
       </c>
       <c r="B14" s="244"/>
-      <c r="C14" s="377" t="s">
+      <c r="C14" s="376" t="s">
         <v>179</v>
       </c>
-      <c r="D14" s="376"/>
-      <c r="E14" s="376"/>
-      <c r="F14" s="376"/>
-      <c r="G14" s="376"/>
-      <c r="H14" s="376"/>
-      <c r="I14" s="376"/>
-      <c r="J14" s="376"/>
-      <c r="K14" s="376"/>
+      <c r="D14" s="375"/>
+      <c r="E14" s="375"/>
+      <c r="F14" s="375"/>
+      <c r="G14" s="375"/>
+      <c r="H14" s="375"/>
+      <c r="I14" s="375"/>
+      <c r="J14" s="375"/>
+      <c r="K14" s="375"/>
       <c r="L14" s="144"/>
       <c r="M14" s="144"/>
       <c r="N14" s="144"/>
@@ -9327,21 +9329,21 @@
       <c r="R14" s="146"/>
     </row>
     <row r="15" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A15" s="374" t="s">
+      <c r="A15" s="373" t="s">
         <v>160</v>
       </c>
       <c r="B15" s="244"/>
-      <c r="C15" s="377" t="s">
+      <c r="C15" s="376" t="s">
         <v>181</v>
       </c>
-      <c r="D15" s="376"/>
-      <c r="E15" s="376"/>
-      <c r="F15" s="376"/>
-      <c r="G15" s="376"/>
-      <c r="H15" s="376"/>
-      <c r="I15" s="376"/>
-      <c r="J15" s="376"/>
-      <c r="K15" s="376"/>
+      <c r="D15" s="375"/>
+      <c r="E15" s="375"/>
+      <c r="F15" s="375"/>
+      <c r="G15" s="375"/>
+      <c r="H15" s="375"/>
+      <c r="I15" s="375"/>
+      <c r="J15" s="375"/>
+      <c r="K15" s="375"/>
       <c r="L15" s="144"/>
       <c r="M15" s="144"/>
       <c r="N15" s="144"/>
@@ -9356,21 +9358,21 @@
       <c r="R15" s="146"/>
     </row>
     <row r="16" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A16" s="374" t="s">
+      <c r="A16" s="373" t="s">
         <v>162</v>
       </c>
       <c r="B16" s="244"/>
-      <c r="C16" s="379" t="s">
+      <c r="C16" s="378" t="s">
         <v>183</v>
       </c>
-      <c r="D16" s="376"/>
-      <c r="E16" s="376"/>
-      <c r="F16" s="376"/>
-      <c r="G16" s="376"/>
-      <c r="H16" s="376"/>
-      <c r="I16" s="376"/>
-      <c r="J16" s="376"/>
-      <c r="K16" s="376"/>
+      <c r="D16" s="375"/>
+      <c r="E16" s="375"/>
+      <c r="F16" s="375"/>
+      <c r="G16" s="375"/>
+      <c r="H16" s="375"/>
+      <c r="I16" s="375"/>
+      <c r="J16" s="375"/>
+      <c r="K16" s="375"/>
       <c r="L16" s="144"/>
       <c r="M16" s="144"/>
       <c r="N16" s="144"/>
@@ -9380,21 +9382,21 @@
       <c r="R16" s="146"/>
     </row>
     <row r="17" spans="1:18" ht="28.5" customHeight="1">
-      <c r="A17" s="374" t="s">
+      <c r="A17" s="373" t="s">
         <v>163</v>
       </c>
       <c r="B17" s="244"/>
-      <c r="C17" s="379" t="s">
+      <c r="C17" s="378" t="s">
         <v>184</v>
       </c>
-      <c r="D17" s="376"/>
-      <c r="E17" s="376"/>
-      <c r="F17" s="376"/>
-      <c r="G17" s="376"/>
-      <c r="H17" s="376"/>
-      <c r="I17" s="376"/>
-      <c r="J17" s="376"/>
-      <c r="K17" s="376"/>
+      <c r="D17" s="375"/>
+      <c r="E17" s="375"/>
+      <c r="F17" s="375"/>
+      <c r="G17" s="375"/>
+      <c r="H17" s="375"/>
+      <c r="I17" s="375"/>
+      <c r="J17" s="375"/>
+      <c r="K17" s="375"/>
       <c r="L17" s="144"/>
       <c r="M17" s="147" t="s">
         <v>185</v>
@@ -9413,21 +9415,21 @@
       <c r="R17" s="146"/>
     </row>
     <row r="18" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A18" s="374" t="s">
+      <c r="A18" s="373" t="s">
         <v>180</v>
       </c>
       <c r="B18" s="244"/>
-      <c r="C18" s="379" t="s">
+      <c r="C18" s="378" t="s">
         <v>187</v>
       </c>
-      <c r="D18" s="376"/>
-      <c r="E18" s="376"/>
-      <c r="F18" s="376"/>
-      <c r="G18" s="376"/>
-      <c r="H18" s="376"/>
-      <c r="I18" s="376"/>
-      <c r="J18" s="376"/>
-      <c r="K18" s="376"/>
+      <c r="D18" s="375"/>
+      <c r="E18" s="375"/>
+      <c r="F18" s="375"/>
+      <c r="G18" s="375"/>
+      <c r="H18" s="375"/>
+      <c r="I18" s="375"/>
+      <c r="J18" s="375"/>
+      <c r="K18" s="375"/>
       <c r="L18" s="144"/>
       <c r="M18" s="147" t="s">
         <v>188</v>
@@ -9441,21 +9443,21 @@
       <c r="R18" s="146"/>
     </row>
     <row r="19" spans="1:18" ht="28.5" customHeight="1">
-      <c r="A19" s="374" t="s">
+      <c r="A19" s="373" t="s">
         <v>182</v>
       </c>
       <c r="B19" s="244"/>
-      <c r="C19" s="379" t="s">
+      <c r="C19" s="378" t="s">
         <v>189</v>
       </c>
-      <c r="D19" s="376"/>
-      <c r="E19" s="376"/>
-      <c r="F19" s="376"/>
-      <c r="G19" s="376"/>
-      <c r="H19" s="376"/>
-      <c r="I19" s="376"/>
-      <c r="J19" s="376"/>
-      <c r="K19" s="376"/>
+      <c r="D19" s="375"/>
+      <c r="E19" s="375"/>
+      <c r="F19" s="375"/>
+      <c r="G19" s="375"/>
+      <c r="H19" s="375"/>
+      <c r="I19" s="375"/>
+      <c r="J19" s="375"/>
+      <c r="K19" s="375"/>
       <c r="L19" s="144"/>
       <c r="M19" s="144"/>
       <c r="N19" s="144"/>
@@ -9470,21 +9472,21 @@
       <c r="R19" s="146"/>
     </row>
     <row r="20" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A20" s="374" t="s">
+      <c r="A20" s="373" t="s">
         <v>164</v>
       </c>
       <c r="B20" s="244"/>
-      <c r="C20" s="379" t="s">
+      <c r="C20" s="378" t="s">
         <v>191</v>
       </c>
-      <c r="D20" s="376"/>
-      <c r="E20" s="376"/>
-      <c r="F20" s="376"/>
-      <c r="G20" s="376"/>
-      <c r="H20" s="376"/>
-      <c r="I20" s="376"/>
-      <c r="J20" s="376"/>
-      <c r="K20" s="376"/>
+      <c r="D20" s="375"/>
+      <c r="E20" s="375"/>
+      <c r="F20" s="375"/>
+      <c r="G20" s="375"/>
+      <c r="H20" s="375"/>
+      <c r="I20" s="375"/>
+      <c r="J20" s="375"/>
+      <c r="K20" s="375"/>
       <c r="L20" s="144"/>
       <c r="M20" s="144"/>
       <c r="N20" s="144"/>
@@ -9499,21 +9501,21 @@
       <c r="R20" s="146"/>
     </row>
     <row r="21" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A21" s="374" t="s">
+      <c r="A21" s="373" t="s">
         <v>186</v>
       </c>
       <c r="B21" s="244"/>
-      <c r="C21" s="379" t="s">
+      <c r="C21" s="378" t="s">
         <v>193</v>
       </c>
-      <c r="D21" s="376"/>
-      <c r="E21" s="376"/>
-      <c r="F21" s="376"/>
-      <c r="G21" s="376"/>
-      <c r="H21" s="376"/>
-      <c r="I21" s="376"/>
-      <c r="J21" s="376"/>
-      <c r="K21" s="376"/>
+      <c r="D21" s="375"/>
+      <c r="E21" s="375"/>
+      <c r="F21" s="375"/>
+      <c r="G21" s="375"/>
+      <c r="H21" s="375"/>
+      <c r="I21" s="375"/>
+      <c r="J21" s="375"/>
+      <c r="K21" s="375"/>
       <c r="L21" s="144"/>
       <c r="M21" s="144"/>
       <c r="N21" s="144"/>
@@ -9528,24 +9530,24 @@
       <c r="R21" s="146"/>
     </row>
     <row r="22" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A22" s="374" t="s">
+      <c r="A22" s="373" t="s">
         <v>192</v>
       </c>
       <c r="B22" s="244"/>
-      <c r="C22" s="378" t="s">
+      <c r="C22" s="377" t="s">
         <v>195</v>
       </c>
-      <c r="D22" s="376"/>
-      <c r="E22" s="376"/>
-      <c r="F22" s="376"/>
-      <c r="G22" s="376"/>
-      <c r="H22" s="376"/>
-      <c r="I22" s="376"/>
-      <c r="J22" s="376"/>
-      <c r="K22" s="376"/>
-      <c r="L22" s="376"/>
-      <c r="M22" s="376"/>
-      <c r="N22" s="376"/>
+      <c r="D22" s="375"/>
+      <c r="E22" s="375"/>
+      <c r="F22" s="375"/>
+      <c r="G22" s="375"/>
+      <c r="H22" s="375"/>
+      <c r="I22" s="375"/>
+      <c r="J22" s="375"/>
+      <c r="K22" s="375"/>
+      <c r="L22" s="375"/>
+      <c r="M22" s="375"/>
+      <c r="N22" s="375"/>
       <c r="O22" s="258"/>
       <c r="P22" s="147" t="s">
         <v>196</v>
@@ -9557,22 +9559,22 @@
       <c r="R22" s="146"/>
     </row>
     <row r="23" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A23" s="374" t="s">
+      <c r="A23" s="373" t="s">
         <v>194</v>
       </c>
       <c r="B23" s="244"/>
-      <c r="C23" s="379" t="s">
+      <c r="C23" s="378" t="s">
         <v>197</v>
       </c>
-      <c r="D23" s="376"/>
-      <c r="E23" s="376"/>
-      <c r="F23" s="376"/>
-      <c r="G23" s="376"/>
-      <c r="H23" s="376"/>
-      <c r="I23" s="376"/>
-      <c r="J23" s="376"/>
-      <c r="K23" s="376"/>
-      <c r="L23" s="376"/>
+      <c r="D23" s="375"/>
+      <c r="E23" s="375"/>
+      <c r="F23" s="375"/>
+      <c r="G23" s="375"/>
+      <c r="H23" s="375"/>
+      <c r="I23" s="375"/>
+      <c r="J23" s="375"/>
+      <c r="K23" s="375"/>
+      <c r="L23" s="375"/>
       <c r="M23" s="144"/>
       <c r="N23" s="144"/>
       <c r="O23" s="144"/>
@@ -9586,22 +9588,22 @@
       <c r="R23" s="146"/>
     </row>
     <row r="24" spans="1:18" ht="30" customHeight="1">
-      <c r="A24" s="374" t="s">
+      <c r="A24" s="373" t="s">
         <v>196</v>
       </c>
       <c r="B24" s="244"/>
-      <c r="C24" s="379" t="s">
+      <c r="C24" s="378" t="s">
         <v>199</v>
       </c>
-      <c r="D24" s="376"/>
-      <c r="E24" s="376"/>
-      <c r="F24" s="376"/>
-      <c r="G24" s="376"/>
-      <c r="H24" s="376"/>
-      <c r="I24" s="376"/>
-      <c r="J24" s="376"/>
-      <c r="K24" s="376"/>
-      <c r="L24" s="376"/>
+      <c r="D24" s="375"/>
+      <c r="E24" s="375"/>
+      <c r="F24" s="375"/>
+      <c r="G24" s="375"/>
+      <c r="H24" s="375"/>
+      <c r="I24" s="375"/>
+      <c r="J24" s="375"/>
+      <c r="K24" s="375"/>
+      <c r="L24" s="375"/>
       <c r="M24" s="144"/>
       <c r="N24" s="144"/>
       <c r="O24" s="144"/>
@@ -9615,21 +9617,21 @@
       <c r="R24" s="146"/>
     </row>
     <row r="25" spans="1:18" ht="14.25" customHeight="1">
-      <c r="A25" s="374" t="s">
+      <c r="A25" s="373" t="s">
         <v>198</v>
       </c>
       <c r="B25" s="244"/>
-      <c r="C25" s="379" t="s">
+      <c r="C25" s="378" t="s">
         <v>201</v>
       </c>
-      <c r="D25" s="376"/>
-      <c r="E25" s="376"/>
-      <c r="F25" s="376"/>
-      <c r="G25" s="376"/>
-      <c r="H25" s="376"/>
-      <c r="I25" s="376"/>
-      <c r="J25" s="376"/>
-      <c r="K25" s="376"/>
+      <c r="D25" s="375"/>
+      <c r="E25" s="375"/>
+      <c r="F25" s="375"/>
+      <c r="G25" s="375"/>
+      <c r="H25" s="375"/>
+      <c r="I25" s="375"/>
+      <c r="J25" s="375"/>
+      <c r="K25" s="375"/>
       <c r="L25" s="144"/>
       <c r="M25" s="144"/>
       <c r="N25" s="144"/>
@@ -9639,21 +9641,21 @@
       <c r="R25" s="146"/>
     </row>
     <row r="26" spans="1:18" ht="15" customHeight="1" thickBot="1">
-      <c r="A26" s="380" t="s">
+      <c r="A26" s="379" t="s">
         <v>202</v>
       </c>
-      <c r="B26" s="381"/>
-      <c r="C26" s="382" t="s">
+      <c r="B26" s="380"/>
+      <c r="C26" s="381" t="s">
         <v>203</v>
       </c>
-      <c r="D26" s="383"/>
-      <c r="E26" s="383"/>
-      <c r="F26" s="383"/>
-      <c r="G26" s="383"/>
-      <c r="H26" s="383"/>
-      <c r="I26" s="383"/>
-      <c r="J26" s="383"/>
-      <c r="K26" s="383"/>
+      <c r="D26" s="382"/>
+      <c r="E26" s="382"/>
+      <c r="F26" s="382"/>
+      <c r="G26" s="382"/>
+      <c r="H26" s="382"/>
+      <c r="I26" s="382"/>
+      <c r="J26" s="382"/>
+      <c r="K26" s="382"/>
       <c r="L26" s="150"/>
       <c r="M26" s="150"/>
       <c r="N26" s="150"/>
@@ -9761,7 +9763,7 @@
   </cols>
   <sheetData>
     <row r="4" spans="3:12">
-      <c r="C4" s="384" t="str">
+      <c r="C4" s="383" t="str">
         <f>'AREA UTIL '!C4</f>
         <v>MATRÍCULA 11.173</v>
       </c>
@@ -9772,7 +9774,7 @@
       <c r="H4" s="248"/>
     </row>
     <row r="5" spans="3:12">
-      <c r="C5" s="384" t="s">
+      <c r="C5" s="383" t="s">
         <v>204</v>
       </c>
       <c r="D5" s="248"/>
@@ -9782,12 +9784,12 @@
       <c r="H5" s="248"/>
     </row>
     <row r="6" spans="3:12">
-      <c r="C6" s="389" t="s">
+      <c r="C6" s="388" t="s">
         <v>190</v>
       </c>
       <c r="D6" s="248"/>
       <c r="E6" s="248"/>
-      <c r="F6" s="386">
+      <c r="F6" s="385">
         <f>'PLANILHA HOMOG'!Q19</f>
         <v>937.24</v>
       </c>
@@ -9795,12 +9797,12 @@
       <c r="H6" s="258"/>
     </row>
     <row r="7" spans="3:12">
-      <c r="C7" s="389" t="s">
+      <c r="C7" s="388" t="s">
         <v>205</v>
       </c>
       <c r="D7" s="248"/>
       <c r="E7" s="248"/>
-      <c r="F7" s="386">
+      <c r="F7" s="385">
         <f>'PLANILHA HOMOG'!Q14</f>
         <v>14159.41</v>
       </c>
@@ -9808,12 +9810,12 @@
       <c r="H7" s="258"/>
     </row>
     <row r="8" spans="3:12">
-      <c r="C8" s="389" t="s">
+      <c r="C8" s="388" t="s">
         <v>206</v>
       </c>
       <c r="D8" s="248"/>
       <c r="E8" s="248"/>
-      <c r="F8" s="386">
+      <c r="F8" s="385">
         <f>'PLANILHA HOMOG'!Q15</f>
         <v>11248.99</v>
       </c>
@@ -9821,12 +9823,12 @@
       <c r="H8" s="258"/>
     </row>
     <row r="9" spans="3:12">
-      <c r="C9" s="389" t="s">
+      <c r="C9" s="388" t="s">
         <v>207</v>
       </c>
       <c r="D9" s="248"/>
       <c r="E9" s="248"/>
-      <c r="F9" s="385">
+      <c r="F9" s="384">
         <v>6</v>
       </c>
       <c r="G9" s="248"/>
@@ -9836,12 +9838,12 @@
       </c>
     </row>
     <row r="10" spans="3:12">
-      <c r="C10" s="389" t="s">
+      <c r="C10" s="388" t="s">
         <v>209</v>
       </c>
       <c r="D10" s="248"/>
       <c r="E10" s="248"/>
-      <c r="F10" s="385">
+      <c r="F10" s="384">
         <v>1</v>
       </c>
       <c r="G10" s="248"/>
@@ -9851,7 +9853,7 @@
       </c>
     </row>
     <row r="11" spans="3:12">
-      <c r="C11" s="389" t="s">
+      <c r="C11" s="388" t="s">
         <v>200</v>
       </c>
       <c r="D11" s="248"/>
@@ -9864,12 +9866,12 @@
       <c r="H11" s="258"/>
     </row>
     <row r="12" spans="3:12">
-      <c r="C12" s="389" t="s">
+      <c r="C12" s="388" t="s">
         <v>210</v>
       </c>
       <c r="D12" s="248"/>
       <c r="E12" s="248"/>
-      <c r="F12" s="385">
+      <c r="F12" s="384">
         <f>'PLANILHA HOMOG'!N18</f>
         <v>0.27100000000000002</v>
       </c>
@@ -9877,12 +9879,12 @@
       <c r="H12" s="258"/>
     </row>
     <row r="13" spans="3:12">
-      <c r="C13" s="389" t="s">
+      <c r="C13" s="388" t="s">
         <v>198</v>
       </c>
       <c r="D13" s="248"/>
       <c r="E13" s="248"/>
-      <c r="F13" s="386">
+      <c r="F13" s="385">
         <f>'PLANILHA HOMOG'!Q23</f>
         <v>253.98</v>
       </c>
@@ -9927,12 +9929,12 @@
       <c r="H16" s="248"/>
     </row>
     <row r="17" spans="3:8">
-      <c r="C17" s="389" t="s">
+      <c r="C17" s="388" t="s">
         <v>213</v>
       </c>
       <c r="D17" s="248"/>
       <c r="E17" s="248"/>
-      <c r="F17" s="385">
+      <c r="F17" s="384">
         <f>AMOSTRAS!E14</f>
         <v>52.034300000000002</v>
       </c>
@@ -9940,12 +9942,12 @@
       <c r="H17" s="258"/>
     </row>
     <row r="18" spans="3:8">
-      <c r="C18" s="389" t="s">
+      <c r="C18" s="388" t="s">
         <v>214</v>
       </c>
       <c r="D18" s="248"/>
       <c r="E18" s="248"/>
-      <c r="F18" s="386">
+      <c r="F18" s="385">
         <f>'PLANILHA HOMOG'!Q17</f>
         <v>13189.81</v>
       </c>
@@ -9953,12 +9955,12 @@
       <c r="H18" s="258"/>
     </row>
     <row r="19" spans="3:8">
-      <c r="C19" s="389" t="s">
+      <c r="C19" s="388" t="s">
         <v>215</v>
       </c>
       <c r="D19" s="248"/>
       <c r="E19" s="248"/>
-      <c r="F19" s="386">
+      <c r="F19" s="385">
         <f>F17*F18</f>
         <v>686322.53048299998</v>
       </c>
@@ -9979,23 +9981,23 @@
       <c r="H20" s="244"/>
     </row>
     <row r="21" spans="3:8">
-      <c r="C21" s="400"/>
+      <c r="C21" s="389"/>
       <c r="D21" s="248"/>
       <c r="E21" s="248"/>
-      <c r="F21" s="387"/>
+      <c r="F21" s="386"/>
       <c r="G21" s="248"/>
       <c r="H21" s="248"/>
     </row>
     <row r="22" spans="3:8">
-      <c r="C22" s="400"/>
+      <c r="C22" s="389"/>
       <c r="D22" s="248"/>
       <c r="E22" s="248"/>
-      <c r="F22" s="387"/>
+      <c r="F22" s="386"/>
       <c r="G22" s="248"/>
       <c r="H22" s="248"/>
     </row>
     <row r="23" spans="3:8">
-      <c r="C23" s="400"/>
+      <c r="C23" s="389"/>
       <c r="D23" s="248"/>
       <c r="E23" s="248"/>
       <c r="F23" s="393"/>
@@ -10013,7 +10015,7 @@
       <c r="H24" s="248"/>
     </row>
     <row r="25" spans="3:8">
-      <c r="C25" s="388" t="s">
+      <c r="C25" s="387" t="s">
         <v>218</v>
       </c>
       <c r="D25" s="248"/>
@@ -10025,19 +10027,19 @@
       <c r="H25" s="258"/>
     </row>
     <row r="26" spans="3:8">
-      <c r="C26" s="388" t="s">
+      <c r="C26" s="387" t="s">
         <v>219</v>
       </c>
       <c r="D26" s="248"/>
       <c r="E26" s="248"/>
-      <c r="F26" s="401">
+      <c r="F26" s="400">
         <v>0.8</v>
       </c>
       <c r="G26" s="248"/>
       <c r="H26" s="258"/>
     </row>
     <row r="27" spans="3:8">
-      <c r="C27" s="388" t="s">
+      <c r="C27" s="387" t="s">
         <v>220</v>
       </c>
       <c r="D27" s="248"/>
@@ -10055,7 +10057,7 @@
       </c>
       <c r="D28" s="243"/>
       <c r="E28" s="243"/>
-      <c r="F28" s="402">
+      <c r="F28" s="401">
         <f>F27</f>
         <v>1600000</v>
       </c>
@@ -10073,12 +10075,12 @@
       <c r="H31" s="248"/>
     </row>
     <row r="32" spans="3:8">
-      <c r="C32" s="389" t="s">
+      <c r="C32" s="388" t="s">
         <v>222</v>
       </c>
       <c r="D32" s="248"/>
       <c r="E32" s="248"/>
-      <c r="F32" s="386">
+      <c r="F32" s="385">
         <f>F20</f>
         <v>686322.53048299998</v>
       </c>
@@ -10086,12 +10088,12 @@
       <c r="H32" s="258"/>
     </row>
     <row r="33" spans="3:8">
-      <c r="C33" s="389" t="s">
+      <c r="C33" s="388" t="s">
         <v>223</v>
       </c>
       <c r="D33" s="248"/>
       <c r="E33" s="248"/>
-      <c r="F33" s="386">
+      <c r="F33" s="385">
         <f>F28</f>
         <v>1600000</v>
       </c>
@@ -10183,7 +10185,7 @@
   </cols>
   <sheetData>
     <row r="5" spans="3:11">
-      <c r="C5" s="384" t="str">
+      <c r="C5" s="383" t="str">
         <f>SANEAMENTO!C4</f>
         <v>MATRÍCULA 11.173</v>
       </c>
@@ -10194,7 +10196,7 @@
       <c r="H5" s="248"/>
     </row>
     <row r="6" spans="3:11">
-      <c r="C6" s="384" t="s">
+      <c r="C6" s="383" t="s">
         <v>225</v>
       </c>
       <c r="D6" s="248"/>
@@ -10204,36 +10206,36 @@
       <c r="H6" s="248"/>
     </row>
     <row r="7" spans="3:11">
-      <c r="C7" s="389" t="s">
+      <c r="C7" s="388" t="s">
         <v>226</v>
       </c>
       <c r="D7" s="248"/>
       <c r="E7" s="248"/>
-      <c r="F7" s="404">
+      <c r="F7" s="403">
         <v>0.13250000000000001</v>
       </c>
       <c r="G7" s="248"/>
       <c r="H7" s="258"/>
     </row>
     <row r="8" spans="3:11">
-      <c r="C8" s="389" t="s">
+      <c r="C8" s="388" t="s">
         <v>227</v>
       </c>
       <c r="D8" s="248"/>
       <c r="E8" s="248"/>
-      <c r="F8" s="385">
+      <c r="F8" s="384">
         <v>36</v>
       </c>
       <c r="G8" s="248"/>
       <c r="H8" s="258"/>
     </row>
     <row r="9" spans="3:11">
-      <c r="C9" s="389" t="s">
+      <c r="C9" s="388" t="s">
         <v>228</v>
       </c>
       <c r="D9" s="248"/>
       <c r="E9" s="248"/>
-      <c r="F9" s="403">
+      <c r="F9" s="402">
         <f>1/((1+F7)^(F8/12))</f>
         <v>0.68847055051621997</v>
       </c>
@@ -10241,12 +10243,12 @@
       <c r="H9" s="258"/>
     </row>
     <row r="10" spans="3:11">
-      <c r="C10" s="389" t="s">
+      <c r="C10" s="388" t="s">
         <v>229</v>
       </c>
       <c r="D10" s="248"/>
       <c r="E10" s="248"/>
-      <c r="F10" s="386">
+      <c r="F10" s="385">
         <f>SANEAMENTO!F20</f>
         <v>686322.53048299998</v>
       </c>
@@ -10282,36 +10284,36 @@
       <c r="K13" s="187"/>
     </row>
     <row r="14" spans="3:11">
-      <c r="C14" s="389" t="s">
+      <c r="C14" s="388" t="s">
         <v>226</v>
       </c>
       <c r="D14" s="248"/>
       <c r="E14" s="248"/>
-      <c r="F14" s="404">
+      <c r="F14" s="403">
         <v>0.12767999999999999</v>
       </c>
       <c r="G14" s="248"/>
       <c r="H14" s="258"/>
     </row>
     <row r="15" spans="3:11">
-      <c r="C15" s="389" t="s">
+      <c r="C15" s="388" t="s">
         <v>227</v>
       </c>
       <c r="D15" s="248"/>
       <c r="E15" s="248"/>
-      <c r="F15" s="385">
+      <c r="F15" s="384">
         <v>36</v>
       </c>
       <c r="G15" s="248"/>
       <c r="H15" s="258"/>
     </row>
     <row r="16" spans="3:11">
-      <c r="C16" s="389" t="s">
+      <c r="C16" s="388" t="s">
         <v>228</v>
       </c>
       <c r="D16" s="248"/>
       <c r="E16" s="248"/>
-      <c r="F16" s="403">
+      <c r="F16" s="402">
         <f>1/((1+F14)^(F15/12))</f>
         <v>0.69733644889224644</v>
       </c>
@@ -10319,12 +10321,12 @@
       <c r="H16" s="258"/>
     </row>
     <row r="17" spans="3:8">
-      <c r="C17" s="389" t="s">
+      <c r="C17" s="388" t="s">
         <v>229</v>
       </c>
       <c r="D17" s="248"/>
       <c r="E17" s="248"/>
-      <c r="F17" s="386">
+      <c r="F17" s="385">
         <f>SANEAMENTO!F28</f>
         <v>1600000</v>
       </c>
@@ -10409,37 +10411,37 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:31" s="68" customFormat="1" ht="17.100000000000001" customHeight="1">
-      <c r="B2" s="405" t="s">
+      <c r="B2" s="404" t="s">
         <v>231</v>
       </c>
-      <c r="C2" s="406"/>
-      <c r="D2" s="406"/>
-      <c r="E2" s="406"/>
-      <c r="F2" s="406"/>
-      <c r="G2" s="406"/>
-      <c r="H2" s="406"/>
-      <c r="I2" s="406"/>
-      <c r="J2" s="406"/>
-      <c r="K2" s="406"/>
-      <c r="L2" s="406"/>
-      <c r="M2" s="406"/>
-      <c r="N2" s="406"/>
-      <c r="O2" s="406"/>
-      <c r="P2" s="406"/>
-      <c r="Q2" s="406"/>
-      <c r="R2" s="406"/>
-      <c r="S2" s="406"/>
-      <c r="T2" s="406"/>
-      <c r="U2" s="406"/>
-      <c r="V2" s="406"/>
-      <c r="W2" s="406"/>
-      <c r="X2" s="406"/>
-      <c r="Y2" s="406"/>
-      <c r="Z2" s="406"/>
-      <c r="AA2" s="406"/>
-      <c r="AB2" s="406"/>
-      <c r="AC2" s="406"/>
-      <c r="AD2" s="406"/>
+      <c r="C2" s="405"/>
+      <c r="D2" s="405"/>
+      <c r="E2" s="405"/>
+      <c r="F2" s="405"/>
+      <c r="G2" s="405"/>
+      <c r="H2" s="405"/>
+      <c r="I2" s="405"/>
+      <c r="J2" s="405"/>
+      <c r="K2" s="405"/>
+      <c r="L2" s="405"/>
+      <c r="M2" s="405"/>
+      <c r="N2" s="405"/>
+      <c r="O2" s="405"/>
+      <c r="P2" s="405"/>
+      <c r="Q2" s="405"/>
+      <c r="R2" s="405"/>
+      <c r="S2" s="405"/>
+      <c r="T2" s="405"/>
+      <c r="U2" s="405"/>
+      <c r="V2" s="405"/>
+      <c r="W2" s="405"/>
+      <c r="X2" s="405"/>
+      <c r="Y2" s="405"/>
+      <c r="Z2" s="405"/>
+      <c r="AA2" s="405"/>
+      <c r="AB2" s="405"/>
+      <c r="AC2" s="405"/>
+      <c r="AD2" s="405"/>
     </row>
     <row r="3" spans="2:31" s="68" customFormat="1" ht="17.100000000000001" customHeight="1">
       <c r="B3" s="69"/>
@@ -10566,39 +10568,39 @@
       <c r="AD9" s="98"/>
     </row>
     <row r="10" spans="2:31" ht="15" customHeight="1">
-      <c r="B10" s="423">
+      <c r="B10" s="422">
         <f>AMOSTRAS!E14</f>
         <v>52.034300000000002</v>
       </c>
-      <c r="C10" s="408"/>
-      <c r="D10" s="408"/>
-      <c r="E10" s="408"/>
-      <c r="F10" s="408"/>
-      <c r="G10" s="408"/>
+      <c r="C10" s="407"/>
+      <c r="D10" s="407"/>
+      <c r="E10" s="407"/>
+      <c r="F10" s="407"/>
+      <c r="G10" s="407"/>
       <c r="H10" s="48" t="s">
         <v>235</v>
       </c>
-      <c r="I10" s="422">
+      <c r="I10" s="421">
         <f>IF(B10=" ","",W11)</f>
         <v>13189.81</v>
       </c>
-      <c r="J10" s="408"/>
-      <c r="K10" s="408"/>
-      <c r="L10" s="408"/>
-      <c r="M10" s="408"/>
-      <c r="N10" s="408"/>
-      <c r="O10" s="408"/>
-      <c r="P10" s="408"/>
+      <c r="J10" s="407"/>
+      <c r="K10" s="407"/>
+      <c r="L10" s="407"/>
+      <c r="M10" s="407"/>
+      <c r="N10" s="407"/>
+      <c r="O10" s="407"/>
+      <c r="P10" s="407"/>
       <c r="Q10" s="48" t="s">
         <v>238</v>
       </c>
-      <c r="R10" s="407">
+      <c r="R10" s="406">
         <f>IF(B10=" ","",I10*B10)</f>
         <v>686322.53048299998</v>
       </c>
-      <c r="S10" s="408"/>
-      <c r="T10" s="408"/>
-      <c r="U10" s="408"/>
+      <c r="S10" s="407"/>
+      <c r="T10" s="407"/>
+      <c r="U10" s="407"/>
       <c r="V10" s="48"/>
       <c r="W10" s="48" t="s">
         <v>239</v>
@@ -10633,13 +10635,13 @@
       <c r="T11" s="48"/>
       <c r="U11" s="99"/>
       <c r="V11" s="48"/>
-      <c r="W11" s="407">
+      <c r="W11" s="406">
         <f>'PLANILHA HOMOG'!Q17</f>
         <v>13189.81</v>
       </c>
-      <c r="X11" s="408"/>
-      <c r="Y11" s="408"/>
-      <c r="Z11" s="408"/>
+      <c r="X11" s="407"/>
+      <c r="Y11" s="407"/>
+      <c r="Z11" s="407"/>
       <c r="AA11" s="48"/>
       <c r="AB11" s="48"/>
       <c r="AC11" s="98"/>
@@ -10666,13 +10668,13 @@
       <c r="Q12" s="48" t="s">
         <v>238</v>
       </c>
-      <c r="R12" s="419">
+      <c r="R12" s="418">
         <f>R10</f>
         <v>686322.53048299998</v>
       </c>
-      <c r="S12" s="408"/>
-      <c r="T12" s="408"/>
-      <c r="U12" s="408"/>
+      <c r="S12" s="407"/>
+      <c r="T12" s="407"/>
+      <c r="U12" s="407"/>
       <c r="V12" s="48"/>
       <c r="W12" s="48"/>
       <c r="X12" s="48"/>
@@ -10692,10 +10694,10 @@
         <v>240</v>
       </c>
       <c r="V14" s="80"/>
-      <c r="W14" s="412"/>
-      <c r="X14" s="408"/>
-      <c r="Y14" s="408"/>
-      <c r="Z14" s="408"/>
+      <c r="W14" s="411"/>
+      <c r="X14" s="407"/>
+      <c r="Y14" s="407"/>
+      <c r="Z14" s="407"/>
       <c r="AA14" s="70"/>
       <c r="AB14" s="70"/>
       <c r="AC14" s="81"/>
@@ -10721,38 +10723,38 @@
       <c r="AD15" s="83"/>
     </row>
     <row r="16" spans="2:31">
-      <c r="B16" s="416" t="s">
+      <c r="B16" s="415" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="408"/>
-      <c r="D16" s="408"/>
-      <c r="E16" s="408"/>
-      <c r="F16" s="408"/>
-      <c r="G16" s="408"/>
+      <c r="C16" s="407"/>
+      <c r="D16" s="407"/>
+      <c r="E16" s="407"/>
+      <c r="F16" s="407"/>
+      <c r="G16" s="407"/>
       <c r="H16" s="67" t="s">
         <v>235</v>
       </c>
-      <c r="I16" s="425" t="str">
+      <c r="I16" s="424" t="str">
         <f>IF(B16=" ","",W11)</f>
         <v/>
       </c>
-      <c r="J16" s="408"/>
-      <c r="K16" s="408"/>
-      <c r="L16" s="408"/>
-      <c r="M16" s="408"/>
-      <c r="N16" s="408"/>
-      <c r="O16" s="408"/>
-      <c r="P16" s="408"/>
+      <c r="J16" s="407"/>
+      <c r="K16" s="407"/>
+      <c r="L16" s="407"/>
+      <c r="M16" s="407"/>
+      <c r="N16" s="407"/>
+      <c r="O16" s="407"/>
+      <c r="P16" s="407"/>
       <c r="Q16" s="67" t="s">
         <v>238</v>
       </c>
-      <c r="R16" s="412" t="str">
+      <c r="R16" s="411" t="str">
         <f>IF(B16=" ","",I16*B16)</f>
         <v/>
       </c>
-      <c r="S16" s="408"/>
-      <c r="T16" s="408"/>
-      <c r="U16" s="408"/>
+      <c r="S16" s="407"/>
+      <c r="T16" s="407"/>
+      <c r="U16" s="407"/>
       <c r="V16" s="80"/>
       <c r="AA16" s="82"/>
       <c r="AB16" s="82"/>
@@ -10764,10 +10766,10 @@
       <c r="S17" s="75"/>
       <c r="U17" s="75"/>
       <c r="V17" s="80"/>
-      <c r="W17" s="412"/>
-      <c r="X17" s="408"/>
-      <c r="Y17" s="408"/>
-      <c r="Z17" s="408"/>
+      <c r="W17" s="411"/>
+      <c r="X17" s="407"/>
+      <c r="Y17" s="407"/>
+      <c r="Z17" s="407"/>
       <c r="AA17" s="82"/>
       <c r="AB17" s="82"/>
       <c r="AC17" s="83"/>
@@ -10791,13 +10793,13 @@
       <c r="Q18" s="67" t="s">
         <v>238</v>
       </c>
-      <c r="R18" s="428" t="str">
+      <c r="R18" s="427" t="str">
         <f>R16</f>
         <v/>
       </c>
-      <c r="S18" s="408"/>
-      <c r="T18" s="408"/>
-      <c r="U18" s="408"/>
+      <c r="S18" s="407"/>
+      <c r="T18" s="407"/>
+      <c r="U18" s="407"/>
       <c r="V18" s="80"/>
       <c r="W18" s="80"/>
       <c r="X18" s="80"/>
@@ -10879,13 +10881,13 @@
       <c r="V22" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W22" s="420">
+      <c r="W22" s="419">
         <f>R12</f>
         <v>686322.53048299998</v>
       </c>
-      <c r="X22" s="415"/>
-      <c r="Y22" s="415"/>
-      <c r="Z22" s="415"/>
+      <c r="X22" s="414"/>
+      <c r="Y22" s="414"/>
+      <c r="Z22" s="414"/>
     </row>
     <row r="23" spans="2:37" s="85" customFormat="1" ht="13.5" customHeight="1">
       <c r="B23" s="85" t="s">
@@ -10894,13 +10896,13 @@
       <c r="V23" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W23" s="414" t="str">
+      <c r="W23" s="413" t="str">
         <f>R16</f>
         <v/>
       </c>
-      <c r="X23" s="415"/>
-      <c r="Y23" s="415"/>
-      <c r="Z23" s="415"/>
+      <c r="X23" s="414"/>
+      <c r="Y23" s="414"/>
+      <c r="Z23" s="414"/>
     </row>
     <row r="24" spans="2:37" s="86" customFormat="1" ht="13.5" customHeight="1">
       <c r="B24" s="86" t="s">
@@ -10909,13 +10911,13 @@
       <c r="V24" s="86" t="s">
         <v>244</v>
       </c>
-      <c r="W24" s="409">
+      <c r="W24" s="408">
         <f>SUM(W22:W23)</f>
         <v>686322.53048299998</v>
       </c>
-      <c r="X24" s="410"/>
-      <c r="Y24" s="410"/>
-      <c r="Z24" s="410"/>
+      <c r="X24" s="409"/>
+      <c r="Y24" s="409"/>
+      <c r="Z24" s="409"/>
     </row>
     <row r="25" spans="2:37" s="85" customFormat="1" ht="13.5" customHeight="1">
       <c r="B25" s="85" t="s">
@@ -10924,13 +10926,13 @@
       <c r="V25" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W25" s="414">
+      <c r="W25" s="413">
         <f>'LAUDO DE AVALIAÇÃO 12-12.4'!H9</f>
         <v>0</v>
       </c>
-      <c r="X25" s="415"/>
-      <c r="Y25" s="415"/>
-      <c r="Z25" s="415"/>
+      <c r="X25" s="414"/>
+      <c r="Y25" s="414"/>
+      <c r="Z25" s="414"/>
     </row>
     <row r="26" spans="2:37" s="85" customFormat="1" ht="13.5" customHeight="1">
       <c r="B26" s="85" t="s">
@@ -10939,13 +10941,13 @@
       <c r="V26" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W26" s="414">
+      <c r="W26" s="413">
         <f>'LAUDO DE AVALIAÇÃO 12-12.4'!H14</f>
         <v>0</v>
       </c>
-      <c r="X26" s="415"/>
-      <c r="Y26" s="415"/>
-      <c r="Z26" s="415"/>
+      <c r="X26" s="414"/>
+      <c r="Y26" s="414"/>
+      <c r="Z26" s="414"/>
     </row>
     <row r="27" spans="2:37" s="85" customFormat="1" ht="13.5" customHeight="1">
       <c r="B27" s="85" t="s">
@@ -10954,13 +10956,13 @@
       <c r="V27" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W27" s="414">
+      <c r="W27" s="413">
         <f>'LAUDO DE AVALIAÇÃO 12-12.4'!H19</f>
         <v>0</v>
       </c>
-      <c r="X27" s="415"/>
-      <c r="Y27" s="415"/>
-      <c r="Z27" s="415"/>
+      <c r="X27" s="414"/>
+      <c r="Y27" s="414"/>
+      <c r="Z27" s="414"/>
     </row>
     <row r="28" spans="2:37" s="85" customFormat="1" ht="13.5" customHeight="1">
       <c r="B28" s="85" t="s">
@@ -10969,13 +10971,13 @@
       <c r="V28" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W28" s="414">
+      <c r="W28" s="413">
         <f>'LAUDO DE AVALIAÇÃO 12-12.4'!H24</f>
         <v>0</v>
       </c>
-      <c r="X28" s="415"/>
-      <c r="Y28" s="415"/>
-      <c r="Z28" s="415"/>
+      <c r="X28" s="414"/>
+      <c r="Y28" s="414"/>
+      <c r="Z28" s="414"/>
     </row>
     <row r="29" spans="2:37" s="85" customFormat="1" ht="13.5" customHeight="1">
       <c r="B29" s="85" t="s">
@@ -10984,13 +10986,13 @@
       <c r="V29" s="85" t="s">
         <v>244</v>
       </c>
-      <c r="W29" s="414">
+      <c r="W29" s="413">
         <f>'LAUDO DE AVALIAÇÃO 13'!G8</f>
         <v>0</v>
       </c>
-      <c r="X29" s="415"/>
-      <c r="Y29" s="415"/>
-      <c r="Z29" s="415"/>
+      <c r="X29" s="414"/>
+      <c r="Y29" s="414"/>
+      <c r="Z29" s="414"/>
     </row>
     <row r="30" spans="2:37" s="86" customFormat="1" ht="13.5" customHeight="1">
       <c r="B30" s="86" t="s">
@@ -10999,13 +11001,13 @@
       <c r="V30" s="86" t="s">
         <v>244</v>
       </c>
-      <c r="W30" s="413">
+      <c r="W30" s="412">
         <f>SUM(W25:Z29)</f>
         <v>0</v>
       </c>
-      <c r="X30" s="410"/>
-      <c r="Y30" s="410"/>
-      <c r="Z30" s="410"/>
+      <c r="X30" s="409"/>
+      <c r="Y30" s="409"/>
+      <c r="Z30" s="409"/>
       <c r="AG30" s="85"/>
     </row>
     <row r="31" spans="2:37" s="86" customFormat="1" ht="13.5" customHeight="1">
@@ -11015,83 +11017,83 @@
       <c r="V31" s="87" t="s">
         <v>244</v>
       </c>
-      <c r="W31" s="418">
+      <c r="W31" s="417">
         <f>W30+W24</f>
         <v>686322.53048299998</v>
       </c>
-      <c r="X31" s="410"/>
-      <c r="Y31" s="410"/>
-      <c r="Z31" s="410"/>
+      <c r="X31" s="409"/>
+      <c r="Y31" s="409"/>
+      <c r="Z31" s="409"/>
       <c r="AG31" s="88"/>
     </row>
     <row r="32" spans="2:37" s="85" customFormat="1" ht="11.25" customHeight="1">
       <c r="B32" s="85" t="s">
         <v>254</v>
       </c>
-      <c r="K32" s="417">
+      <c r="K32" s="416">
         <v>43009</v>
       </c>
-      <c r="L32" s="415"/>
-      <c r="M32" s="415"/>
-      <c r="N32" s="415"/>
-      <c r="O32" s="415"/>
-      <c r="P32" s="415"/>
-      <c r="Q32" s="415"/>
-      <c r="R32" s="415"/>
-      <c r="S32" s="415"/>
-      <c r="T32" s="415"/>
-      <c r="U32" s="415"/>
-      <c r="V32" s="415"/>
-      <c r="W32" s="415"/>
-      <c r="X32" s="415"/>
-      <c r="Y32" s="415"/>
-      <c r="Z32" s="415"/>
+      <c r="L32" s="414"/>
+      <c r="M32" s="414"/>
+      <c r="N32" s="414"/>
+      <c r="O32" s="414"/>
+      <c r="P32" s="414"/>
+      <c r="Q32" s="414"/>
+      <c r="R32" s="414"/>
+      <c r="S32" s="414"/>
+      <c r="T32" s="414"/>
+      <c r="U32" s="414"/>
+      <c r="V32" s="414"/>
+      <c r="W32" s="414"/>
+      <c r="X32" s="414"/>
+      <c r="Y32" s="414"/>
+      <c r="Z32" s="414"/>
       <c r="AG32" s="88"/>
     </row>
     <row r="33" spans="2:37" s="86" customFormat="1" ht="17.25" customHeight="1">
-      <c r="O33" s="429" t="s">
+      <c r="O33" s="428" t="s">
         <v>255</v>
       </c>
-      <c r="P33" s="410"/>
-      <c r="Q33" s="410"/>
-      <c r="R33" s="410"/>
-      <c r="S33" s="410"/>
-      <c r="T33" s="410"/>
-      <c r="U33" s="410"/>
-      <c r="V33" s="410"/>
-      <c r="W33" s="430" t="s">
+      <c r="P33" s="409"/>
+      <c r="Q33" s="409"/>
+      <c r="R33" s="409"/>
+      <c r="S33" s="409"/>
+      <c r="T33" s="409"/>
+      <c r="U33" s="409"/>
+      <c r="V33" s="409"/>
+      <c r="W33" s="429" t="s">
         <v>256</v>
       </c>
-      <c r="X33" s="321"/>
-      <c r="Y33" s="321"/>
-      <c r="Z33" s="321"/>
-      <c r="AA33" s="321"/>
-      <c r="AB33" s="321"/>
-      <c r="AC33" s="321"/>
-      <c r="AD33" s="321"/>
+      <c r="X33" s="320"/>
+      <c r="Y33" s="320"/>
+      <c r="Z33" s="320"/>
+      <c r="AA33" s="320"/>
+      <c r="AB33" s="320"/>
+      <c r="AC33" s="320"/>
+      <c r="AD33" s="320"/>
       <c r="AG33" s="89"/>
     </row>
     <row r="34" spans="2:37" s="85" customFormat="1" ht="19.5" customHeight="1">
       <c r="O34" s="48"/>
       <c r="P34" s="48"/>
-      <c r="Q34" s="421">
+      <c r="Q34" s="420">
         <f>W31*0.9</f>
         <v>617690.27743470005</v>
       </c>
-      <c r="R34" s="415"/>
-      <c r="S34" s="415"/>
-      <c r="T34" s="415"/>
+      <c r="R34" s="414"/>
+      <c r="S34" s="414"/>
+      <c r="T34" s="414"/>
       <c r="U34" s="48"/>
       <c r="V34" s="48"/>
       <c r="W34" s="48"/>
       <c r="X34" s="48"/>
-      <c r="Y34" s="421">
+      <c r="Y34" s="420">
         <f>W31*1.1</f>
         <v>754954.78353130003</v>
       </c>
-      <c r="Z34" s="415"/>
-      <c r="AA34" s="415"/>
-      <c r="AB34" s="415"/>
+      <c r="Z34" s="414"/>
+      <c r="AA34" s="414"/>
+      <c r="AB34" s="414"/>
       <c r="AC34" s="48"/>
       <c r="AD34" s="48"/>
       <c r="AG34" s="86"/>
@@ -11154,32 +11156,32 @@
     </row>
     <row r="37" spans="2:37" ht="10.5" customHeight="1"/>
     <row r="38" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B38" s="411"/>
-      <c r="C38" s="408"/>
+      <c r="B38" s="410"/>
+      <c r="C38" s="407"/>
     </row>
     <row r="39" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B39" s="411"/>
-      <c r="C39" s="408"/>
+      <c r="B39" s="410"/>
+      <c r="C39" s="407"/>
     </row>
     <row r="40" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B40" s="411"/>
-      <c r="C40" s="408"/>
+      <c r="B40" s="410"/>
+      <c r="C40" s="407"/>
     </row>
     <row r="41" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B41" s="411"/>
-      <c r="C41" s="408"/>
+      <c r="B41" s="410"/>
+      <c r="C41" s="407"/>
     </row>
     <row r="42" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B42" s="411"/>
-      <c r="C42" s="408"/>
+      <c r="B42" s="410"/>
+      <c r="C42" s="407"/>
     </row>
     <row r="43" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B43" s="411"/>
-      <c r="C43" s="408"/>
+      <c r="B43" s="410"/>
+      <c r="C43" s="407"/>
     </row>
     <row r="44" spans="2:37" ht="14.25" customHeight="1">
-      <c r="B44" s="411"/>
-      <c r="C44" s="408"/>
+      <c r="B44" s="410"/>
+      <c r="C44" s="407"/>
     </row>
     <row r="45" spans="2:37" ht="15" customHeight="1">
       <c r="B45" s="96"/>
@@ -11250,10 +11252,10 @@
     </row>
     <row r="48" spans="2:37" ht="14.25" customHeight="1"/>
     <row r="49" spans="5:16" ht="13.5" customHeight="1">
-      <c r="E49" s="427"/>
-      <c r="F49" s="408"/>
-      <c r="G49" s="408"/>
-      <c r="H49" s="408"/>
+      <c r="E49" s="426"/>
+      <c r="F49" s="407"/>
+      <c r="G49" s="407"/>
+      <c r="H49" s="407"/>
       <c r="I49" s="91"/>
       <c r="J49" s="91"/>
       <c r="K49" s="91"/>
@@ -11276,40 +11278,40 @@
     </row>
     <row r="51" spans="5:16" ht="11.25" customHeight="1"/>
     <row r="52" spans="5:16" ht="14.25" customHeight="1">
-      <c r="H52" s="424"/>
-      <c r="I52" s="321"/>
-      <c r="J52" s="321"/>
-      <c r="K52" s="321"/>
-      <c r="L52" s="321"/>
-      <c r="M52" s="321"/>
-      <c r="N52" s="321"/>
-      <c r="O52" s="321"/>
-      <c r="P52" s="321"/>
+      <c r="H52" s="423"/>
+      <c r="I52" s="320"/>
+      <c r="J52" s="320"/>
+      <c r="K52" s="320"/>
+      <c r="L52" s="320"/>
+      <c r="M52" s="320"/>
+      <c r="N52" s="320"/>
+      <c r="O52" s="320"/>
+      <c r="P52" s="320"/>
     </row>
     <row r="53" spans="5:16" ht="6.75" customHeight="1"/>
     <row r="54" spans="5:16" ht="12.75" customHeight="1"/>
     <row r="55" spans="5:16" ht="13.5" customHeight="1">
-      <c r="H55" s="426"/>
-      <c r="I55" s="321"/>
-      <c r="J55" s="321"/>
-      <c r="K55" s="321"/>
-      <c r="L55" s="321"/>
-      <c r="M55" s="321"/>
-      <c r="N55" s="321"/>
-      <c r="O55" s="321"/>
-      <c r="P55" s="321"/>
+      <c r="H55" s="425"/>
+      <c r="I55" s="320"/>
+      <c r="J55" s="320"/>
+      <c r="K55" s="320"/>
+      <c r="L55" s="320"/>
+      <c r="M55" s="320"/>
+      <c r="N55" s="320"/>
+      <c r="O55" s="320"/>
+      <c r="P55" s="320"/>
     </row>
     <row r="56" spans="5:16" ht="4.5" customHeight="1"/>
     <row r="57" spans="5:16" ht="14.25" customHeight="1">
-      <c r="H57" s="424"/>
-      <c r="I57" s="321"/>
-      <c r="J57" s="321"/>
-      <c r="K57" s="321"/>
-      <c r="L57" s="321"/>
-      <c r="M57" s="321"/>
-      <c r="N57" s="321"/>
-      <c r="O57" s="321"/>
-      <c r="P57" s="321"/>
+      <c r="H57" s="423"/>
+      <c r="I57" s="320"/>
+      <c r="J57" s="320"/>
+      <c r="K57" s="320"/>
+      <c r="L57" s="320"/>
+      <c r="M57" s="320"/>
+      <c r="N57" s="320"/>
+      <c r="O57" s="320"/>
+      <c r="P57" s="320"/>
     </row>
     <row r="58" spans="5:16" ht="6.75" customHeight="1"/>
   </sheetData>

</xml_diff>